<commit_message>
Project architecture work & small document changes
Small correction in UserStories
Small updates to ProjectPlan
Added 8 empty classes of entities to the java project
Removed empty test class
Implemented architecture for Customer class
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A00327279\Documents\GitHub\Software-Engineering-Project-G1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Downloads\GitRepositories\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF54CD4D-BC42-4CF8-82BB-4438ABBD08D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98740330-EDCD-4F3B-BF22-E68E8C5CB1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
+    <workbookView xWindow="-28920" yWindow="-1020" windowWidth="29040" windowHeight="15720" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -155,15 +155,6 @@
     <t>I want to create a customer</t>
   </si>
   <si>
-    <t>Verify that a valid customer createress can be entered</t>
-  </si>
-  <si>
-    <t>Verify that, if all entered values are valid, the Customers name, createress and phone number are updated on the database</t>
-  </si>
-  <si>
-    <t>Verify that the customers createress is printed to the screen</t>
-  </si>
-  <si>
     <t>I want to have a specialised login for the system</t>
   </si>
   <si>
@@ -570,13 +561,22 @@
   </si>
   <si>
     <t>I want to delete</t>
+  </si>
+  <si>
+    <t>Verify that the customers address is printed to the screen</t>
+  </si>
+  <si>
+    <t>Verify that a valid customer address can be entered</t>
+  </si>
+  <si>
+    <t>Verify that, if all entered values are valid, the Customers name, address and phone number are updated on the database</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,7 +653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -688,35 +688,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1053,43 +1050,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
   <dimension ref="A1:J179"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="1.625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="80.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="180.875" style="20" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="1.5703125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="80.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="180.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="0" style="2" hidden="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.125" style="2"/>
+    <col min="6" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="16" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="16"/>
       <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="15">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="2" t="s">
         <v>22</v>
       </c>
       <c r="E3" s="1"/>
@@ -1099,12 +1096,12 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="15">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="C4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E4" s="1"/>
@@ -1114,12 +1111,12 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="15">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="1"/>
@@ -1129,10 +1126,10 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="15">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E6" s="1"/>
@@ -1142,10 +1139,10 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" ht="15">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="1"/>
@@ -1155,7 +1152,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="15">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="C8" s="5"/>
       <c r="E8" s="1"/>
@@ -1165,14 +1162,14 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10" ht="15">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>2</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="1"/>
@@ -1182,12 +1179,12 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10" ht="15">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="C10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="E10" s="1"/>
@@ -1197,12 +1194,12 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10" ht="15">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="C11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E11" s="1"/>
@@ -1212,10 +1209,10 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="1:10" ht="15">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E12" s="1"/>
@@ -1225,10 +1222,10 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:10" ht="15">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E13" s="1"/>
@@ -1238,19 +1235,19 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="15">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>3</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="20" t="s">
-        <v>44</v>
+      <c r="D15" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1258,13 +1255,13 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:10" ht="15">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="C16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>45</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -1272,13 +1269,13 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" ht="15">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="C17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>46</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1286,7 +1283,7 @@
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" ht="15">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="9"/>
       <c r="C18" s="5"/>
       <c r="E18" s="1"/>
@@ -1295,15 +1292,15 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9" ht="15">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>4</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="20" t="s">
-        <v>54</v>
+      <c r="D19" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -1311,10 +1308,10 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" ht="15">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="C20" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1322,10 +1319,10 @@
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9" ht="15">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="C21" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -1333,7 +1330,7 @@
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" ht="15">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="C22" s="5"/>
       <c r="E22" s="1"/>
@@ -1342,11 +1339,11 @@
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:9" ht="15">
-      <c r="A23" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B23" s="13"/>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="16"/>
       <c r="C23" s="5"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1354,15 +1351,15 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" ht="15">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>1</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -1370,13 +1367,13 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:9" ht="15">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="C25" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>45</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -1384,13 +1381,13 @@
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:9" ht="15">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="C26" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D26" s="20" t="s">
         <v>46</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1398,7 +1395,7 @@
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" spans="1:9" ht="15">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
       <c r="C27" s="5"/>
       <c r="E27" s="1"/>
@@ -1407,15 +1404,15 @@
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:9" ht="15">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>2</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>51</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -1423,13 +1420,13 @@
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" ht="30">
+    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
       <c r="C29" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -1437,13 +1434,13 @@
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" ht="15">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="C30" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D30" s="20" t="s">
-        <v>58</v>
+        <v>53</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -1451,11 +1448,11 @@
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" ht="15">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
       <c r="C31" s="5"/>
-      <c r="D31" s="20" t="s">
-        <v>55</v>
+      <c r="D31" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -1463,7 +1460,7 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9" ht="15">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="C32" s="5"/>
       <c r="E32" s="1"/>
@@ -1472,15 +1469,15 @@
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9" ht="15">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>3</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>62</v>
+        <v>45</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -1488,13 +1485,13 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" ht="15">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
       <c r="C34" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>63</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -1502,10 +1499,10 @@
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
     </row>
-    <row r="35" spans="1:9" ht="15">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="C35" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -1513,7 +1510,7 @@
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="1:9" ht="15">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="C36" s="5"/>
       <c r="E36" s="1"/>
@@ -1522,15 +1519,15 @@
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" ht="15">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="9">
         <v>4</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D37" s="20" t="s">
-        <v>68</v>
+        <v>45</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -1538,13 +1535,13 @@
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9" ht="15">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
       <c r="C38" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>69</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -1552,13 +1549,13 @@
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9" ht="15">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="C39" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>70</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -1566,11 +1563,11 @@
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
     </row>
-    <row r="40" spans="1:9" ht="15">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="C40" s="5"/>
-      <c r="D40" s="20" t="s">
-        <v>71</v>
+      <c r="D40" s="2" t="s">
+        <v>68</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
@@ -1578,11 +1575,11 @@
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
     </row>
-    <row r="41" spans="1:9" ht="15">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="C41" s="5"/>
-      <c r="D41" s="20" t="s">
-        <v>72</v>
+      <c r="D41" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -1590,11 +1587,11 @@
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
     </row>
-    <row r="42" spans="1:9" ht="15">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="C42" s="5"/>
-      <c r="D42" s="20" t="s">
-        <v>73</v>
+      <c r="D42" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -1602,7 +1599,7 @@
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
     </row>
-    <row r="43" spans="1:9" ht="15">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="C43" s="5"/>
       <c r="E43" s="1"/>
@@ -1611,11 +1608,11 @@
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
     </row>
-    <row r="44" spans="1:9" ht="15">
-      <c r="A44" s="18" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B44" s="19"/>
+      <c r="B44" s="20"/>
       <c r="C44" s="5"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -1623,7 +1620,7 @@
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
     </row>
-    <row r="45" spans="1:9" ht="15">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>1</v>
       </c>
@@ -1639,13 +1636,13 @@
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
     </row>
-    <row r="46" spans="1:9" ht="15">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="C46" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>39</v>
+        <v>176</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -1653,13 +1650,13 @@
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
     </row>
-    <row r="47" spans="1:9" ht="15">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
       <c r="C47" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -1667,11 +1664,11 @@
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="1:9" ht="15">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
       <c r="C48" s="5"/>
       <c r="D48" s="8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -1679,7 +1676,7 @@
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" spans="1:9" ht="15">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
       <c r="C49" s="5"/>
       <c r="D49" s="8" t="s">
@@ -1691,11 +1688,11 @@
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="1:9" ht="15">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
       <c r="C50" s="5"/>
       <c r="D50" s="8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -1703,7 +1700,7 @@
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
     </row>
-    <row r="51" spans="1:9" ht="15">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
       <c r="C51" s="5"/>
       <c r="D51" s="8" t="s">
@@ -1715,7 +1712,7 @@
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" spans="1:9" ht="15">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -1723,7 +1720,7 @@
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
     </row>
-    <row r="53" spans="1:9" ht="15">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="9">
         <v>2</v>
       </c>
@@ -1739,7 +1736,7 @@
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
     </row>
-    <row r="54" spans="1:9" ht="15">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
       <c r="C54" s="6" t="s">
         <v>8</v>
@@ -1753,7 +1750,7 @@
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
     </row>
-    <row r="55" spans="1:9" ht="15">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
       <c r="C55" s="6" t="s">
         <v>9</v>
@@ -1767,7 +1764,7 @@
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
     </row>
-    <row r="56" spans="1:9" ht="15">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
       <c r="C56" s="5"/>
       <c r="D56" s="8" t="s">
@@ -1779,7 +1776,7 @@
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
     </row>
-    <row r="57" spans="1:9" ht="15">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
       <c r="C57" s="5"/>
       <c r="D57" s="8" t="s">
@@ -1791,7 +1788,7 @@
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
     </row>
-    <row r="58" spans="1:9" ht="15">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="C58" s="5"/>
       <c r="E58" s="1"/>
@@ -1800,14 +1797,14 @@
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
     </row>
-    <row r="59" spans="1:9" ht="15">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="9">
         <v>3</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D59" s="20" t="s">
+      <c r="D59" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E59" s="1"/>
@@ -1816,7 +1813,7 @@
       <c r="H59" s="1"/>
       <c r="I59" s="1"/>
     </row>
-    <row r="60" spans="1:9" ht="15">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
       <c r="C60" s="6" t="s">
         <v>10</v>
@@ -1830,10 +1827,10 @@
       <c r="H60" s="1"/>
       <c r="I60" s="1"/>
     </row>
-    <row r="61" spans="1:9" ht="15">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="9"/>
       <c r="C61" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>6</v>
@@ -1844,11 +1841,11 @@
       <c r="H61" s="1"/>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" spans="1:9" ht="15">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="9"/>
       <c r="C62" s="5"/>
       <c r="D62" s="8" t="s">
-        <v>39</v>
+        <v>176</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
@@ -1856,7 +1853,7 @@
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
     </row>
-    <row r="63" spans="1:9" ht="15">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
       <c r="C63" s="5"/>
       <c r="D63" s="8" t="s">
@@ -1868,7 +1865,7 @@
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
     </row>
-    <row r="64" spans="1:9" ht="15">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="9"/>
       <c r="C64" s="5"/>
       <c r="D64" s="8" t="s">
@@ -1880,11 +1877,11 @@
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
     </row>
-    <row r="65" spans="1:9" ht="15">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="9"/>
       <c r="C65" s="5"/>
       <c r="D65" s="8" t="s">
-        <v>40</v>
+        <v>177</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -1892,7 +1889,7 @@
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
     </row>
-    <row r="66" spans="1:9" ht="15">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="C66" s="5"/>
       <c r="E66" s="1"/>
@@ -1901,14 +1898,14 @@
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
     </row>
-    <row r="67" spans="1:9" ht="15">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="9">
         <v>4</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D67" s="20" t="s">
+      <c r="D67" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E67" s="1"/>
@@ -1917,13 +1914,13 @@
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
     </row>
-    <row r="68" spans="1:9" ht="15">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
       <c r="B68" s="7"/>
       <c r="C68" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="D68" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E68" s="1"/>
@@ -1932,7 +1929,7 @@
       <c r="H68" s="1"/>
       <c r="I68" s="1"/>
     </row>
-    <row r="69" spans="1:9" ht="15">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
       <c r="B69" s="7"/>
       <c r="C69" s="6" t="s">
@@ -1947,11 +1944,11 @@
       <c r="H69" s="1"/>
       <c r="I69" s="1"/>
     </row>
-    <row r="70" spans="1:9" ht="15">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="9"/>
       <c r="C70" s="5"/>
       <c r="D70" s="8" t="s">
-        <v>41</v>
+        <v>175</v>
       </c>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
@@ -1959,7 +1956,7 @@
       <c r="H70" s="1"/>
       <c r="I70" s="1"/>
     </row>
-    <row r="71" spans="1:9" ht="15">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="9"/>
       <c r="C71" s="5"/>
       <c r="D71" s="8" t="s">
@@ -1971,7 +1968,7 @@
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
     </row>
-    <row r="72" spans="1:9" ht="15">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="9"/>
       <c r="C72" s="5"/>
       <c r="E72" s="1"/>
@@ -1980,11 +1977,11 @@
       <c r="H72" s="1"/>
       <c r="I72" s="1"/>
     </row>
-    <row r="73" spans="1:9" ht="15">
-      <c r="A73" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B73" s="13"/>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73" s="16"/>
       <c r="C73" s="5"/>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
@@ -1992,7 +1989,7 @@
       <c r="H73" s="1"/>
       <c r="I73" s="1"/>
     </row>
-    <row r="74" spans="1:9" ht="15">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="9">
         <v>1</v>
       </c>
@@ -2000,7 +1997,7 @@
         <v>4</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
@@ -2008,13 +2005,13 @@
       <c r="H74" s="1"/>
       <c r="I74" s="1"/>
     </row>
-    <row r="75" spans="1:9" ht="15">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="9"/>
       <c r="C75" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
@@ -2022,13 +2019,13 @@
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
     </row>
-    <row r="76" spans="1:9" ht="15">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="9"/>
       <c r="C76" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
@@ -2036,11 +2033,11 @@
       <c r="H76" s="1"/>
       <c r="I76" s="1"/>
     </row>
-    <row r="77" spans="1:9" ht="15">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="9"/>
       <c r="C77" s="5"/>
       <c r="D77" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
@@ -2048,11 +2045,11 @@
       <c r="H77" s="1"/>
       <c r="I77" s="1"/>
     </row>
-    <row r="78" spans="1:9" ht="15">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="9"/>
       <c r="C78" s="5"/>
       <c r="D78" s="8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
@@ -2060,11 +2057,11 @@
       <c r="H78" s="1"/>
       <c r="I78" s="1"/>
     </row>
-    <row r="79" spans="1:9" ht="15">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
       <c r="C79" s="5"/>
       <c r="D79" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
@@ -2072,7 +2069,7 @@
       <c r="H79" s="1"/>
       <c r="I79" s="1"/>
     </row>
-    <row r="80" spans="1:9" ht="15">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
       <c r="C80" s="5"/>
       <c r="E80" s="1"/>
@@ -2081,7 +2078,7 @@
       <c r="H80" s="1"/>
       <c r="I80" s="1"/>
     </row>
-    <row r="81" spans="1:9" ht="15">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="9">
         <v>2</v>
       </c>
@@ -2089,7 +2086,7 @@
         <v>4</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
@@ -2097,13 +2094,13 @@
       <c r="H81" s="1"/>
       <c r="I81" s="1"/>
     </row>
-    <row r="82" spans="1:9" ht="15">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="9"/>
       <c r="C82" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
@@ -2111,13 +2108,13 @@
       <c r="H82" s="1"/>
       <c r="I82" s="1"/>
     </row>
-    <row r="83" spans="1:9" ht="15">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
       <c r="C83" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
@@ -2125,11 +2122,11 @@
       <c r="H83" s="1"/>
       <c r="I83" s="1"/>
     </row>
-    <row r="84" spans="1:9" ht="15">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="9"/>
       <c r="C84" s="5"/>
       <c r="D84" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
@@ -2137,7 +2134,7 @@
       <c r="H84" s="1"/>
       <c r="I84" s="1"/>
     </row>
-    <row r="85" spans="1:9" ht="15">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
       <c r="C85" s="5"/>
       <c r="D85" s="8" t="s">
@@ -2149,7 +2146,7 @@
       <c r="H85" s="1"/>
       <c r="I85" s="1"/>
     </row>
-    <row r="86" spans="1:9" ht="15">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
       <c r="C86" s="5"/>
       <c r="E86" s="1"/>
@@ -2158,7 +2155,7 @@
       <c r="H86" s="1"/>
       <c r="I86" s="1"/>
     </row>
-    <row r="87" spans="1:9" ht="15">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="9">
         <v>3</v>
       </c>
@@ -2166,7 +2163,7 @@
         <v>4</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
@@ -2174,13 +2171,13 @@
       <c r="H87" s="1"/>
       <c r="I87" s="1"/>
     </row>
-    <row r="88" spans="1:9" ht="15">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
       <c r="C88" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
@@ -2188,13 +2185,13 @@
       <c r="H88" s="1"/>
       <c r="I88" s="1"/>
     </row>
-    <row r="89" spans="1:9" ht="15">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
       <c r="C89" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
@@ -2202,7 +2199,7 @@
       <c r="H89" s="1"/>
       <c r="I89" s="1"/>
     </row>
-    <row r="90" spans="1:9" ht="15">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
       <c r="C90" s="5"/>
       <c r="D90" s="8" t="s">
@@ -2214,11 +2211,11 @@
       <c r="H90" s="1"/>
       <c r="I90" s="1"/>
     </row>
-    <row r="91" spans="1:9" ht="15">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
       <c r="C91" s="5"/>
       <c r="D91" s="8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
@@ -2226,11 +2223,11 @@
       <c r="H91" s="1"/>
       <c r="I91" s="1"/>
     </row>
-    <row r="92" spans="1:9" ht="15">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
       <c r="C92" s="5"/>
       <c r="D92" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
@@ -2238,11 +2235,11 @@
       <c r="H92" s="1"/>
       <c r="I92" s="1"/>
     </row>
-    <row r="93" spans="1:9" ht="15">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="9"/>
       <c r="C93" s="5"/>
       <c r="D93" s="8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
@@ -2250,11 +2247,11 @@
       <c r="H93" s="1"/>
       <c r="I93" s="1"/>
     </row>
-    <row r="94" spans="1:9" ht="15">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="9"/>
       <c r="C94" s="5"/>
       <c r="D94" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -2262,7 +2259,7 @@
       <c r="H94" s="1"/>
       <c r="I94" s="1"/>
     </row>
-    <row r="95" spans="1:9" ht="15">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
       <c r="C95" s="5"/>
       <c r="E95" s="1"/>
@@ -2271,7 +2268,7 @@
       <c r="H95" s="1"/>
       <c r="I95" s="1"/>
     </row>
-    <row r="96" spans="1:9" ht="15">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="9">
         <v>4</v>
       </c>
@@ -2279,7 +2276,7 @@
         <v>4</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
@@ -2287,13 +2284,13 @@
       <c r="H96" s="1"/>
       <c r="I96" s="1"/>
     </row>
-    <row r="97" spans="1:9" ht="15">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="9"/>
       <c r="C97" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D97" s="8" t="s">
         <v>95</v>
-      </c>
-      <c r="D97" s="8" t="s">
-        <v>98</v>
       </c>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
@@ -2301,13 +2298,13 @@
       <c r="H97" s="1"/>
       <c r="I97" s="1"/>
     </row>
-    <row r="98" spans="1:9" ht="15">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
       <c r="C98" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D98" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="D98" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
@@ -2315,11 +2312,11 @@
       <c r="H98" s="1"/>
       <c r="I98" s="1"/>
     </row>
-    <row r="99" spans="1:9" ht="15">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="9"/>
       <c r="C99" s="5"/>
       <c r="D99" s="8" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
@@ -2327,11 +2324,11 @@
       <c r="H99" s="1"/>
       <c r="I99" s="1"/>
     </row>
-    <row r="100" spans="1:9" ht="15">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
       <c r="C100" s="5"/>
-      <c r="D100" s="20" t="s">
-        <v>101</v>
+      <c r="D100" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
@@ -2339,11 +2336,11 @@
       <c r="H100" s="1"/>
       <c r="I100" s="1"/>
     </row>
-    <row r="101" spans="1:9" ht="15">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="9"/>
       <c r="C101" s="5"/>
-      <c r="D101" s="20" t="s">
-        <v>102</v>
+      <c r="D101" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
@@ -2351,11 +2348,11 @@
       <c r="H101" s="1"/>
       <c r="I101" s="1"/>
     </row>
-    <row r="102" spans="1:9" ht="15">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="9"/>
       <c r="C102" s="5"/>
       <c r="D102" s="8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
@@ -2363,11 +2360,11 @@
       <c r="H102" s="1"/>
       <c r="I102" s="1"/>
     </row>
-    <row r="103" spans="1:9" ht="15">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="9"/>
       <c r="C103" s="5"/>
       <c r="D103" s="8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
@@ -2375,7 +2372,7 @@
       <c r="H103" s="1"/>
       <c r="I103" s="1"/>
     </row>
-    <row r="104" spans="1:9" ht="15">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="9"/>
       <c r="C104" s="5"/>
       <c r="E104" s="1"/>
@@ -2384,11 +2381,11 @@
       <c r="H104" s="1"/>
       <c r="I104" s="1"/>
     </row>
-    <row r="105" spans="1:9" ht="15">
-      <c r="A105" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="B105" s="13"/>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B105" s="16"/>
       <c r="C105" s="5"/>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
@@ -2396,15 +2393,15 @@
       <c r="H105" s="1"/>
       <c r="I105" s="1"/>
     </row>
-    <row r="106" spans="1:9" ht="15">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="9">
         <v>1</v>
       </c>
       <c r="C106" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D106" s="20" t="s">
-        <v>108</v>
+      <c r="D106" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
@@ -2412,13 +2409,13 @@
       <c r="H106" s="1"/>
       <c r="I106" s="1"/>
     </row>
-    <row r="107" spans="1:9" ht="15">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="9"/>
       <c r="C107" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D107" s="20" t="s">
-        <v>109</v>
+        <v>104</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
@@ -2426,13 +2423,13 @@
       <c r="H107" s="1"/>
       <c r="I107" s="1"/>
     </row>
-    <row r="108" spans="1:9" ht="15">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="9"/>
       <c r="C108" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D108" s="20" t="s">
-        <v>114</v>
+      <c r="D108" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
@@ -2440,7 +2437,7 @@
       <c r="H108" s="1"/>
       <c r="I108" s="1"/>
     </row>
-    <row r="109" spans="1:9" ht="15">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="9"/>
       <c r="C109" s="5"/>
       <c r="E109" s="1"/>
@@ -2449,15 +2446,15 @@
       <c r="H109" s="1"/>
       <c r="I109" s="1"/>
     </row>
-    <row r="110" spans="1:9" ht="15">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="9">
         <v>2</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D110" s="20" t="s">
-        <v>113</v>
+      <c r="D110" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
@@ -2465,13 +2462,13 @@
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
     </row>
-    <row r="111" spans="1:9" ht="15">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="9"/>
       <c r="C111" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D111" s="20" t="s">
-        <v>86</v>
+        <v>108</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
@@ -2479,13 +2476,13 @@
       <c r="H111" s="1"/>
       <c r="I111" s="1"/>
     </row>
-    <row r="112" spans="1:9" ht="15">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="9"/>
       <c r="C112" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D112" s="21" t="s">
-        <v>119</v>
+        <v>109</v>
+      </c>
+      <c r="D112" s="14" t="s">
+        <v>116</v>
       </c>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
@@ -2493,11 +2490,11 @@
       <c r="H112" s="1"/>
       <c r="I112" s="1"/>
     </row>
-    <row r="113" spans="1:9" ht="15">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="9"/>
       <c r="C113" s="5"/>
-      <c r="D113" s="20" t="s">
-        <v>115</v>
+      <c r="D113" s="2" t="s">
+        <v>112</v>
       </c>
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
@@ -2505,7 +2502,7 @@
       <c r="H113" s="1"/>
       <c r="I113" s="1"/>
     </row>
-    <row r="114" spans="1:9" ht="15">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="9"/>
       <c r="C114" s="5"/>
       <c r="E114" s="1"/>
@@ -2514,15 +2511,15 @@
       <c r="H114" s="1"/>
       <c r="I114" s="1"/>
     </row>
-    <row r="115" spans="1:9" ht="15">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="9">
         <v>3</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D115" s="20" t="s">
-        <v>118</v>
+      <c r="D115" s="2" t="s">
+        <v>115</v>
       </c>
       <c r="E115" s="1"/>
       <c r="F115" s="1"/>
@@ -2530,13 +2527,13 @@
       <c r="H115" s="1"/>
       <c r="I115" s="1"/>
     </row>
-    <row r="116" spans="1:9" ht="15">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="9"/>
       <c r="C116" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="D116" s="20" t="s">
-        <v>86</v>
+        <v>113</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
@@ -2544,13 +2541,13 @@
       <c r="H116" s="1"/>
       <c r="I116" s="1"/>
     </row>
-    <row r="117" spans="1:9" ht="15">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="9"/>
       <c r="C117" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D117" s="20" t="s">
-        <v>119</v>
+        <v>114</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>116</v>
       </c>
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
@@ -2558,11 +2555,11 @@
       <c r="H117" s="1"/>
       <c r="I117" s="1"/>
     </row>
-    <row r="118" spans="1:9" ht="15">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="9"/>
       <c r="C118" s="5"/>
-      <c r="D118" s="20" t="s">
-        <v>120</v>
+      <c r="D118" s="2" t="s">
+        <v>117</v>
       </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
@@ -2570,11 +2567,11 @@
       <c r="H118" s="1"/>
       <c r="I118" s="1"/>
     </row>
-    <row r="119" spans="1:9" ht="15">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="9"/>
       <c r="C119" s="5"/>
-      <c r="D119" s="20" t="s">
-        <v>121</v>
+      <c r="D119" s="2" t="s">
+        <v>118</v>
       </c>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
@@ -2582,11 +2579,11 @@
       <c r="H119" s="1"/>
       <c r="I119" s="1"/>
     </row>
-    <row r="120" spans="1:9" ht="15">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="9"/>
       <c r="C120" s="5"/>
-      <c r="D120" s="20" t="s">
-        <v>122</v>
+      <c r="D120" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
@@ -2594,7 +2591,7 @@
       <c r="H120" s="1"/>
       <c r="I120" s="1"/>
     </row>
-    <row r="121" spans="1:9" ht="15">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="9"/>
       <c r="C121" s="5"/>
       <c r="E121" s="1"/>
@@ -2603,15 +2600,15 @@
       <c r="H121" s="1"/>
       <c r="I121" s="1"/>
     </row>
-    <row r="122" spans="1:9" ht="15">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="9">
         <v>4</v>
       </c>
       <c r="C122" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D122" s="20" t="s">
-        <v>125</v>
+      <c r="D122" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
@@ -2619,13 +2616,13 @@
       <c r="H122" s="1"/>
       <c r="I122" s="1"/>
     </row>
-    <row r="123" spans="1:9" ht="15">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="9"/>
       <c r="C123" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D123" s="20" t="s">
-        <v>86</v>
+        <v>120</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
@@ -2633,13 +2630,13 @@
       <c r="H123" s="1"/>
       <c r="I123" s="1"/>
     </row>
-    <row r="124" spans="1:9" ht="15">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="9"/>
       <c r="C124" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D124" s="20" t="s">
-        <v>126</v>
+        <v>121</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
@@ -2647,11 +2644,11 @@
       <c r="H124" s="1"/>
       <c r="I124" s="1"/>
     </row>
-    <row r="125" spans="1:9" ht="15">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="9"/>
       <c r="C125" s="5"/>
-      <c r="D125" s="20" t="s">
-        <v>127</v>
+      <c r="D125" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
@@ -2659,7 +2656,7 @@
       <c r="H125" s="1"/>
       <c r="I125" s="1"/>
     </row>
-    <row r="126" spans="1:9" ht="15">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="9"/>
       <c r="C126" s="5"/>
       <c r="E126" s="1"/>
@@ -2668,9 +2665,9 @@
       <c r="H126" s="1"/>
       <c r="I126" s="1"/>
     </row>
-    <row r="127" spans="1:9" ht="15">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C127" s="5"/>
       <c r="E127" s="1"/>
@@ -2679,15 +2676,15 @@
       <c r="H127" s="1"/>
       <c r="I127" s="1"/>
     </row>
-    <row r="128" spans="1:9" ht="15">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="9">
         <v>1</v>
       </c>
       <c r="C128" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D128" s="20" t="s">
-        <v>143</v>
+      <c r="D128" s="2" t="s">
+        <v>140</v>
       </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
@@ -2695,10 +2692,10 @@
       <c r="H128" s="1"/>
       <c r="I128" s="1"/>
     </row>
-    <row r="129" spans="1:9" ht="15">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="9"/>
       <c r="C129" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
@@ -2706,10 +2703,10 @@
       <c r="H129" s="1"/>
       <c r="I129" s="1"/>
     </row>
-    <row r="130" spans="1:9" ht="15">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="9"/>
       <c r="C130" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
@@ -2717,358 +2714,358 @@
       <c r="H130" s="1"/>
       <c r="I130" s="1"/>
     </row>
-    <row r="131" spans="1:9">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="9"/>
       <c r="C131" s="4"/>
     </row>
-    <row r="132" spans="1:9" ht="15">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="9">
         <v>2</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D132" s="8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="133" spans="1:9" ht="15">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="9"/>
       <c r="C133" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="134" spans="1:9" ht="15">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="9"/>
       <c r="C134" s="6" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D134" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="135" spans="1:9" ht="15">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="9"/>
       <c r="C135" s="4"/>
       <c r="D135" s="8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="136" spans="1:9" ht="15">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="9"/>
       <c r="C136" s="4"/>
       <c r="D136" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="137" spans="1:9">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="9"/>
       <c r="C137" s="4"/>
     </row>
-    <row r="138" spans="1:9" ht="15">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="9">
         <v>3</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D138" s="8" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="139" spans="1:9" ht="30">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A139" s="9"/>
       <c r="C139" s="6" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D139" s="8" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="140" spans="1:9" ht="15">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="11"/>
       <c r="B140" s="8"/>
       <c r="C140" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D140" s="8"/>
     </row>
-    <row r="141" spans="1:9">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="9"/>
       <c r="C141" s="4"/>
     </row>
-    <row r="142" spans="1:9">
-      <c r="A142" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="B142" s="13"/>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B142" s="16"/>
       <c r="C142" s="4"/>
     </row>
-    <row r="143" spans="1:9" ht="15">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="9">
         <v>1</v>
       </c>
       <c r="C143" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D143" s="8" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="144" spans="1:9" ht="15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="9"/>
       <c r="C144" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D144" s="8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" ht="15">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="9"/>
       <c r="C145" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D145" s="8"/>
     </row>
-    <row r="146" spans="1:4">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="9"/>
       <c r="C146" s="4"/>
     </row>
-    <row r="147" spans="1:4" ht="15">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="9">
         <v>2</v>
       </c>
       <c r="C147" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D147" s="8" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" ht="15">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="9"/>
       <c r="C148" s="6" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D148" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" ht="15">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="9"/>
       <c r="C149" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D149" s="8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" ht="15">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="9"/>
       <c r="C150" s="4"/>
       <c r="D150" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" ht="15">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="9"/>
       <c r="C151" s="4"/>
       <c r="D151" s="8" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="9"/>
       <c r="C152" s="4"/>
     </row>
-    <row r="153" spans="1:4" ht="15">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="9">
         <v>3</v>
       </c>
       <c r="C153" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D153" s="8" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" ht="15">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="11"/>
       <c r="B154" s="8"/>
       <c r="C154" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D154" s="8"/>
     </row>
-    <row r="155" spans="1:4" ht="15">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="11"/>
       <c r="B155" s="8"/>
       <c r="C155" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D155" s="8"/>
     </row>
-    <row r="156" spans="1:4">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="9"/>
       <c r="C156" s="4"/>
     </row>
-    <row r="157" spans="1:4" ht="15">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="9">
         <v>4</v>
       </c>
       <c r="C157" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D157" s="8" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" ht="15">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="9"/>
       <c r="C158" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D158" s="8" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" ht="15">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="9"/>
       <c r="C159" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D159" s="8"/>
     </row>
-    <row r="160" spans="1:4">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="9"/>
       <c r="C160" s="4"/>
     </row>
-    <row r="161" spans="1:4">
-      <c r="A161" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="B161" s="13"/>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B161" s="16"/>
       <c r="C161" s="4"/>
     </row>
-    <row r="162" spans="1:4" ht="15">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="9">
         <v>1</v>
       </c>
       <c r="C162" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D162" s="8" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" ht="15">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="9"/>
       <c r="C163" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D163" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" ht="15">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="9"/>
       <c r="C164" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D164" s="8" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="9"/>
       <c r="C165" s="4"/>
     </row>
-    <row r="166" spans="1:4" ht="15">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="9">
         <v>2</v>
       </c>
       <c r="C166" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D166" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="D166" s="8" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" ht="15">
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="9"/>
       <c r="C167" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" ht="15">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="9"/>
       <c r="C168" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" ht="15">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
         <v>3</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D170" s="8"/>
     </row>
-    <row r="171" spans="1:4" ht="15">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="8"/>
       <c r="B171" s="8"/>
       <c r="C171" s="3" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D171" s="8"/>
     </row>
-    <row r="172" spans="1:4" ht="15">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="8"/>
       <c r="B172" s="8"/>
       <c r="C172" s="3"/>
       <c r="D172" s="8"/>
     </row>
-    <row r="174" spans="1:4" ht="15">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
         <v>4</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D174" s="8"/>
     </row>
-    <row r="175" spans="1:4" ht="15">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C175" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D175" s="8"/>
     </row>
-    <row r="176" spans="1:4" ht="15">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C176" s="3"/>
       <c r="D176" s="8"/>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
         <v>5</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C179" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
small update adding first + last names to customer
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Downloads\GitRepositories\Software-Engineering-Project-G1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89e05dc7f8bbc142/Documents/GitHub/Software-Engineering-Project-G1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98740330-EDCD-4F3B-BF22-E68E8C5CB1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{98740330-EDCD-4F3B-BF22-E68E8C5CB1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C5930A-661F-4325-A644-1182943C4B14}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1020" windowWidth="29040" windowHeight="15720" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="181">
   <si>
     <t>Number</t>
   </si>
@@ -56,9 +56,6 @@
     <t>so that I can expand my business</t>
   </si>
   <si>
-    <t>Verify that a valid(3-50 characters) customer name can be entered</t>
-  </si>
-  <si>
     <t>verify that a valid(only integers) customer phone number can be entered</t>
   </si>
   <si>
@@ -224,9 +221,6 @@
     <t>Verify that a valid(greater than one, matches an existing area code) area code can be entered</t>
   </si>
   <si>
-    <t>Verify that a valid(only integers) customer phone number can be entered</t>
-  </si>
-  <si>
     <t>I want to mark whether deliveries on the given day were successful or not</t>
   </si>
   <si>
@@ -554,9 +548,6 @@
     <t>Verify that when a delivery is not marked as successful, it is rescheduled to a later date</t>
   </si>
   <si>
-    <t>I want to create</t>
-  </si>
-  <si>
     <t>I want to read</t>
   </si>
   <si>
@@ -570,6 +561,24 @@
   </si>
   <si>
     <t>Verify that, if all entered values are valid, the Customers name, address and phone number are updated on the database</t>
+  </si>
+  <si>
+    <t>Verify that a valid(1 or more characters) customer first name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(1 or more characters) customer last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(10 numbers) customer phone number can be entered</t>
+  </si>
+  <si>
+    <t>I want to create a delivery docket</t>
+  </si>
+  <si>
+    <t>so that my delivery people can know what deliveries need to be made on a given day</t>
+  </si>
+  <si>
+    <t>Verify that all orders on the order database are entered onto the delivery docket, including the order ID, order date, customer ID, customer address, customer name and order item</t>
   </si>
 </sst>
 </file>
@@ -653,7 +662,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -703,16 +712,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1049,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
-  <dimension ref="A1:J179"/>
+  <dimension ref="A1:J182"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
@@ -1061,10 +1079,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="22"/>
       <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
@@ -1073,10 +1091,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="16"/>
+      <c r="A2" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="20"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -1087,7 +1105,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1099,10 +1117,10 @@
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="C4" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -1117,7 +1135,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1130,7 +1148,7 @@
       <c r="A6" s="9"/>
       <c r="C6" s="5"/>
       <c r="D6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1143,7 +1161,7 @@
       <c r="A7" s="9"/>
       <c r="C7" s="5"/>
       <c r="D7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1170,7 +1188,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1182,10 +1200,10 @@
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="C10" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1197,10 +1215,10 @@
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="C11" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1213,7 +1231,7 @@
       <c r="A12" s="9"/>
       <c r="C12" s="5"/>
       <c r="D12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -1226,7 +1244,7 @@
       <c r="A13" s="9"/>
       <c r="C13" s="5"/>
       <c r="D13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -1247,7 +1265,7 @@
         <v>4</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1258,10 +1276,10 @@
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="C16" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -1272,10 +1290,10 @@
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="C17" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1284,8 +1302,6 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
-      <c r="C18" s="5"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -1293,15 +1309,8 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
-        <v>4</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="A19" s="9"/>
+      <c r="C19" s="5"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -1309,9 +1318,14 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
+      <c r="A20" s="9">
+        <v>4</v>
+      </c>
       <c r="C20" s="5" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1322,7 +1336,7 @@
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="C21" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -1332,7 +1346,9 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
-      <c r="C22" s="5"/>
+      <c r="C22" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -1340,10 +1356,7 @@
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" s="16"/>
+      <c r="A23" s="9"/>
       <c r="C23" s="5"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1352,15 +1365,11 @@
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="9">
-        <v>1</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="A24" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="16"/>
+      <c r="C24" s="5"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -1368,12 +1377,14 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
+      <c r="A25" s="9">
+        <v>1</v>
+      </c>
       <c r="C25" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -1384,10 +1395,10 @@
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
       <c r="C26" s="5" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1397,7 +1408,12 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
-      <c r="C27" s="5"/>
+      <c r="C27" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -1405,28 +1421,23 @@
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="9">
-        <v>2</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A28" s="9"/>
+      <c r="C28" s="5"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="9">
+        <v>2</v>
+      </c>
       <c r="C29" s="5" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -1434,13 +1445,13 @@
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
       <c r="C30" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -1450,9 +1461,11 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
-      <c r="C31" s="5"/>
+      <c r="C31" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="D31" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -1463,6 +1476,9 @@
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="C32" s="5"/>
+      <c r="D32" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
@@ -1470,15 +1486,8 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="9">
-        <v>3</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>59</v>
-      </c>
+      <c r="A33" s="9"/>
+      <c r="C33" s="5"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -1486,12 +1495,14 @@
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="9"/>
+      <c r="A34" s="9">
+        <v>3</v>
+      </c>
       <c r="C34" s="5" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -1502,7 +1513,10 @@
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
       <c r="C35" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -1512,7 +1526,9 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
-      <c r="C36" s="5"/>
+      <c r="C36" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
@@ -1520,15 +1536,8 @@
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="9">
-        <v>4</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="A37" s="9"/>
+      <c r="C37" s="5"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -1536,12 +1545,14 @@
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="9"/>
+      <c r="A38" s="9">
+        <v>4</v>
+      </c>
       <c r="C38" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -1552,10 +1563,10 @@
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="C39" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -1565,9 +1576,11 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
-      <c r="C40" s="5"/>
+      <c r="C40" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="D40" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
@@ -1579,7 +1592,7 @@
       <c r="A41" s="9"/>
       <c r="C41" s="5"/>
       <c r="D41" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -1591,7 +1604,7 @@
       <c r="A42" s="9"/>
       <c r="C42" s="5"/>
       <c r="D42" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -1602,6 +1615,9 @@
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="C43" s="5"/>
+      <c r="D43" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
@@ -1609,10 +1625,7 @@
       <c r="I43" s="1"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B44" s="20"/>
+      <c r="A44" s="9"/>
       <c r="C44" s="5"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -1621,15 +1634,11 @@
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="9">
-        <v>1</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>6</v>
-      </c>
+      <c r="A45" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="5"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
@@ -1637,12 +1646,14 @@
       <c r="I45" s="1"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="9"/>
+      <c r="A46" s="9">
+        <v>1</v>
+      </c>
       <c r="C46" s="6" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -1651,12 +1662,11 @@
       <c r="I46" s="1"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="9"/>
       <c r="C47" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>62</v>
+        <v>37</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -1666,9 +1676,11 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
-      <c r="C48" s="5"/>
+      <c r="C48" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="D48" s="8" t="s">
-        <v>61</v>
+        <v>173</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -1678,9 +1690,8 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-      <c r="C49" s="5"/>
       <c r="D49" s="8" t="s">
-        <v>14</v>
+        <v>177</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -1692,7 +1703,7 @@
       <c r="A50" s="9"/>
       <c r="C50" s="5"/>
       <c r="D50" s="8" t="s">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -1704,7 +1715,7 @@
       <c r="A51" s="9"/>
       <c r="C51" s="5"/>
       <c r="D51" s="8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -1714,6 +1725,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="8" t="s">
+        <v>105</v>
+      </c>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
@@ -1721,14 +1736,10 @@
       <c r="I52" s="1"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="9">
-        <v>2</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="A53" s="9"/>
+      <c r="C53" s="5"/>
       <c r="D53" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -1738,12 +1749,6 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
-      <c r="C54" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>13</v>
-      </c>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
@@ -1751,12 +1756,14 @@
       <c r="I54" s="1"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="9"/>
+      <c r="A55" s="9">
+        <v>2</v>
+      </c>
       <c r="C55" s="6" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -1766,9 +1773,11 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
-      <c r="C56" s="5"/>
+      <c r="C56" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="D56" s="8" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -1778,9 +1787,11 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
-      <c r="C57" s="5"/>
+      <c r="C57" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="D57" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -1791,6 +1802,9 @@
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="C58" s="5"/>
+      <c r="D58" s="8" t="s">
+        <v>33</v>
+      </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
@@ -1798,14 +1812,10 @@
       <c r="I58" s="1"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="9">
-        <v>3</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>15</v>
+      <c r="A59" s="9"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="8" t="s">
+        <v>34</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
@@ -1815,12 +1825,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
-      <c r="C60" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>13</v>
-      </c>
+      <c r="C60" s="5"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
@@ -1828,12 +1833,14 @@
       <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="9"/>
+      <c r="A61" s="9">
+        <v>3</v>
+      </c>
       <c r="C61" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
@@ -1843,9 +1850,11 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="9"/>
-      <c r="C62" s="5"/>
+      <c r="C62" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="D62" s="8" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
@@ -1855,9 +1864,11 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="9"/>
-      <c r="C63" s="5"/>
+      <c r="C63" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="D63" s="8" t="s">
-        <v>7</v>
+        <v>175</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -1866,10 +1877,8 @@
       <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="9"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="8" t="s">
-        <v>14</v>
+      <c r="D64" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
@@ -1881,7 +1890,7 @@
       <c r="A65" s="9"/>
       <c r="C65" s="5"/>
       <c r="D65" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -1892,6 +1901,9 @@
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
       <c r="C66" s="5"/>
+      <c r="D66" s="8" t="s">
+        <v>6</v>
+      </c>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
@@ -1899,14 +1911,10 @@
       <c r="I66" s="1"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" s="9">
-        <v>4</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>15</v>
+      <c r="A67" s="9"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="8" t="s">
+        <v>13</v>
       </c>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
@@ -1915,13 +1923,10 @@
       <c r="I67" s="1"/>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A68" s="10"/>
-      <c r="B68" s="7"/>
-      <c r="C68" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>20</v>
+      <c r="A68" s="9"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="8" t="s">
+        <v>174</v>
       </c>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
@@ -1930,14 +1935,8 @@
       <c r="I68" s="1"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" s="10"/>
-      <c r="B69" s="7"/>
-      <c r="C69" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>18</v>
-      </c>
+      <c r="A69" s="9"/>
+      <c r="C69" s="5"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
@@ -1945,10 +1944,14 @@
       <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" s="9"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="8" t="s">
-        <v>175</v>
+      <c r="A70" s="9">
+        <v>4</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
@@ -1957,9 +1960,12 @@
       <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="9"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="8" t="s">
+      <c r="A71" s="10"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E71" s="1"/>
@@ -1969,8 +1975,14 @@
       <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A72" s="9"/>
-      <c r="C72" s="5"/>
+      <c r="A72" s="10"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>17</v>
+      </c>
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
@@ -1978,11 +1990,11 @@
       <c r="I72" s="1"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B73" s="16"/>
+      <c r="A73" s="9"/>
       <c r="C73" s="5"/>
+      <c r="D73" s="8" t="s">
+        <v>172</v>
+      </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
       <c r="G73" s="1"/>
@@ -1990,14 +2002,10 @@
       <c r="I73" s="1"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74" s="9">
-        <v>1</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A74" s="9"/>
+      <c r="C74" s="5"/>
       <c r="D74" s="8" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
@@ -2007,12 +2015,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="9"/>
-      <c r="C75" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>77</v>
-      </c>
+      <c r="C75" s="5"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
@@ -2020,13 +2023,11 @@
       <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="9"/>
-      <c r="C76" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>75</v>
-      </c>
+      <c r="A76" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B76" s="23"/>
+      <c r="C76" s="5"/>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
@@ -2034,10 +2035,14 @@
       <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="9"/>
-      <c r="C77" s="5"/>
+      <c r="A77" s="9">
+        <v>1</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D77" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
@@ -2047,9 +2052,11 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="9"/>
-      <c r="C78" s="5"/>
+      <c r="C78" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="D78" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
@@ -2059,9 +2066,11 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
-      <c r="C79" s="5"/>
+      <c r="C79" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="D79" s="8" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
@@ -2072,6 +2081,9 @@
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
       <c r="C80" s="5"/>
+      <c r="D80" s="8" t="s">
+        <v>74</v>
+      </c>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
       <c r="G80" s="1"/>
@@ -2079,14 +2091,10 @@
       <c r="I80" s="1"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="9">
-        <v>2</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A81" s="9"/>
+      <c r="C81" s="5"/>
       <c r="D81" s="8" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
@@ -2096,11 +2104,9 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="9"/>
-      <c r="C82" s="5" t="s">
+      <c r="C82" s="5"/>
+      <c r="D82" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>83</v>
       </c>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
@@ -2110,12 +2116,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
-      <c r="C83" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>84</v>
-      </c>
+      <c r="C83" s="5"/>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
@@ -2123,10 +2124,14 @@
       <c r="I83" s="1"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="9"/>
-      <c r="C84" s="5"/>
+      <c r="A84" s="9">
+        <v>2</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D84" s="8" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
@@ -2136,9 +2141,11 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
-      <c r="C85" s="5"/>
+      <c r="C85" s="5" t="s">
+        <v>77</v>
+      </c>
       <c r="D85" s="8" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
@@ -2148,7 +2155,12 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
-      <c r="C86" s="5"/>
+      <c r="C86" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>82</v>
+      </c>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
@@ -2156,14 +2168,10 @@
       <c r="I86" s="1"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="9">
-        <v>3</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A87" s="9"/>
+      <c r="C87" s="5"/>
       <c r="D87" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
@@ -2173,11 +2181,9 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
-      <c r="C88" s="5" t="s">
-        <v>86</v>
-      </c>
+      <c r="C88" s="5"/>
       <c r="D88" s="8" t="s">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
@@ -2187,12 +2193,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
-      <c r="C89" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D89" s="8" t="s">
-        <v>84</v>
-      </c>
+      <c r="C89" s="5"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
@@ -2200,10 +2201,14 @@
       <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="9"/>
-      <c r="C90" s="5"/>
+      <c r="A90" s="9">
+        <v>3</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D90" s="8" t="s">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
@@ -2213,9 +2218,11 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
-      <c r="C91" s="5"/>
+      <c r="C91" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="D91" s="8" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
@@ -2225,9 +2232,11 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
-      <c r="C92" s="5"/>
+      <c r="C92" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="D92" s="8" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
@@ -2239,7 +2248,7 @@
       <c r="A93" s="9"/>
       <c r="C93" s="5"/>
       <c r="D93" s="8" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
@@ -2251,7 +2260,7 @@
       <c r="A94" s="9"/>
       <c r="C94" s="5"/>
       <c r="D94" s="8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -2262,6 +2271,9 @@
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
       <c r="C95" s="5"/>
+      <c r="D95" s="8" t="s">
+        <v>86</v>
+      </c>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
@@ -2269,14 +2281,10 @@
       <c r="I95" s="1"/>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" s="9">
-        <v>4</v>
-      </c>
-      <c r="C96" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A96" s="9"/>
+      <c r="C96" s="5"/>
       <c r="D96" s="8" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
@@ -2286,11 +2294,9 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="9"/>
-      <c r="C97" s="5" t="s">
-        <v>92</v>
-      </c>
+      <c r="C97" s="5"/>
       <c r="D97" s="8" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
@@ -2300,12 +2306,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
-      <c r="C98" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D98" s="8" t="s">
-        <v>96</v>
-      </c>
+      <c r="C98" s="5"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
       <c r="G98" s="1"/>
@@ -2313,10 +2314,14 @@
       <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="9"/>
-      <c r="C99" s="5"/>
+      <c r="A99" s="9">
+        <v>4</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D99" s="8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
@@ -2326,9 +2331,11 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="2" t="s">
-        <v>98</v>
+      <c r="C100" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D100" s="8" t="s">
+        <v>93</v>
       </c>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
@@ -2338,9 +2345,11 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="9"/>
-      <c r="C101" s="5"/>
-      <c r="D101" s="2" t="s">
-        <v>99</v>
+      <c r="C101" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>94</v>
       </c>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
@@ -2352,7 +2361,7 @@
       <c r="A102" s="9"/>
       <c r="C102" s="5"/>
       <c r="D102" s="8" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
@@ -2363,8 +2372,8 @@
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="9"/>
       <c r="C103" s="5"/>
-      <c r="D103" s="8" t="s">
-        <v>101</v>
+      <c r="D103" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
@@ -2375,6 +2384,9 @@
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="9"/>
       <c r="C104" s="5"/>
+      <c r="D104" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="E104" s="1"/>
       <c r="F104" s="1"/>
       <c r="G104" s="1"/>
@@ -2382,11 +2394,11 @@
       <c r="I104" s="1"/>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A105" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="B105" s="16"/>
+      <c r="A105" s="9"/>
       <c r="C105" s="5"/>
+      <c r="D105" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
       <c r="G105" s="1"/>
@@ -2394,14 +2406,10 @@
       <c r="I105" s="1"/>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A106" s="9">
-        <v>1</v>
-      </c>
-      <c r="C106" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>105</v>
+      <c r="A106" s="9"/>
+      <c r="C106" s="5"/>
+      <c r="D106" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
@@ -2411,12 +2419,7 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="9"/>
-      <c r="C107" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>106</v>
-      </c>
+      <c r="C107" s="5"/>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
@@ -2424,13 +2427,11 @@
       <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A108" s="9"/>
-      <c r="C108" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>111</v>
-      </c>
+      <c r="A108" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B108" s="23"/>
+      <c r="C108" s="5"/>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
@@ -2438,8 +2439,15 @@
       <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" s="9"/>
-      <c r="C109" s="5"/>
+      <c r="A109" s="9">
+        <v>1</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
       <c r="G109" s="1"/>
@@ -2447,14 +2455,12 @@
       <c r="I109" s="1"/>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A110" s="9">
-        <v>2</v>
-      </c>
+      <c r="A110" s="9"/>
       <c r="C110" s="5" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
@@ -2465,10 +2471,10 @@
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="9"/>
       <c r="C111" s="5" t="s">
-        <v>108</v>
+        <v>5</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
@@ -2478,12 +2484,7 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="9"/>
-      <c r="C112" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D112" s="14" t="s">
-        <v>116</v>
-      </c>
+      <c r="C112" s="5"/>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
@@ -2491,10 +2492,14 @@
       <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="9"/>
-      <c r="C113" s="5"/>
+      <c r="A113" s="9">
+        <v>2</v>
+      </c>
+      <c r="C113" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D113" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
@@ -2504,7 +2509,12 @@
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="9"/>
-      <c r="C114" s="5"/>
+      <c r="C114" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="E114" s="1"/>
       <c r="F114" s="1"/>
       <c r="G114" s="1"/>
@@ -2512,14 +2522,12 @@
       <c r="I114" s="1"/>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A115" s="9">
-        <v>3</v>
-      </c>
+      <c r="A115" s="9"/>
       <c r="C115" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>115</v>
+        <v>107</v>
+      </c>
+      <c r="D115" s="14" t="s">
+        <v>114</v>
       </c>
       <c r="E115" s="1"/>
       <c r="F115" s="1"/>
@@ -2529,11 +2537,9 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="9"/>
-      <c r="C116" s="5" t="s">
-        <v>113</v>
-      </c>
+      <c r="C116" s="5"/>
       <c r="D116" s="2" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
@@ -2543,12 +2549,7 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="9"/>
-      <c r="C117" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>116</v>
-      </c>
+      <c r="C117" s="5"/>
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
@@ -2556,10 +2557,14 @@
       <c r="I117" s="1"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" s="9"/>
-      <c r="C118" s="5"/>
+      <c r="A118" s="9">
+        <v>3</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D118" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
@@ -2569,9 +2574,11 @@
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="9"/>
-      <c r="C119" s="5"/>
+      <c r="C119" s="5" t="s">
+        <v>111</v>
+      </c>
       <c r="D119" s="2" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
@@ -2581,9 +2588,11 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="9"/>
-      <c r="C120" s="5"/>
+      <c r="C120" s="5" t="s">
+        <v>112</v>
+      </c>
       <c r="D120" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
@@ -2594,6 +2603,9 @@
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="9"/>
       <c r="C121" s="5"/>
+      <c r="D121" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
@@ -2601,14 +2613,10 @@
       <c r="I121" s="1"/>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="9">
-        <v>4</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A122" s="9"/>
+      <c r="C122" s="5"/>
       <c r="D122" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
@@ -2618,11 +2626,9 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="9"/>
-      <c r="C123" s="5" t="s">
-        <v>120</v>
-      </c>
+      <c r="C123" s="5"/>
       <c r="D123" s="2" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
@@ -2632,12 +2638,7 @@
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="9"/>
-      <c r="C124" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>123</v>
-      </c>
+      <c r="C124" s="5"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
       <c r="G124" s="1"/>
@@ -2645,10 +2646,14 @@
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="9"/>
-      <c r="C125" s="5"/>
+      <c r="A125" s="9">
+        <v>4</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D125" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
@@ -2658,7 +2663,12 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="9"/>
-      <c r="C126" s="5"/>
+      <c r="C126" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
       <c r="G126" s="1"/>
@@ -2666,10 +2676,13 @@
       <c r="I126" s="1"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A127" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C127" s="5"/>
+      <c r="A127" s="9"/>
+      <c r="C127" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>121</v>
+      </c>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
@@ -2677,14 +2690,10 @@
       <c r="I127" s="1"/>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A128" s="9">
-        <v>1</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A128" s="9"/>
+      <c r="C128" s="5"/>
       <c r="D128" s="2" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
@@ -2694,9 +2703,7 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="9"/>
-      <c r="C129" s="5" t="s">
-        <v>127</v>
-      </c>
+      <c r="C129" s="5"/>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
@@ -2704,10 +2711,10 @@
       <c r="I129" s="1"/>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A130" s="9"/>
-      <c r="C130" s="5" t="s">
-        <v>126</v>
-      </c>
+      <c r="A130" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C130" s="5"/>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
@@ -2715,369 +2722,390 @@
       <c r="I130" s="1"/>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" s="9"/>
-      <c r="C131" s="4"/>
+      <c r="A131" s="9">
+        <v>1</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A132" s="9">
-        <v>2</v>
-      </c>
-      <c r="C132" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D132" s="8" t="s">
-        <v>136</v>
+      <c r="A132" s="9"/>
+      <c r="C132" s="5" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="9"/>
-      <c r="C133" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D133" s="8" t="s">
-        <v>130</v>
+      <c r="C133" s="5" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="9"/>
-      <c r="C134" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D134" s="8" t="s">
-        <v>137</v>
-      </c>
+      <c r="C134" s="4"/>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A135" s="9"/>
-      <c r="C135" s="4"/>
+      <c r="A135" s="9">
+        <v>2</v>
+      </c>
+      <c r="C135" s="6" t="s">
+        <v>126</v>
+      </c>
       <c r="D135" s="8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="9"/>
-      <c r="C136" s="4"/>
+      <c r="C136" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="D136" s="8" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="9"/>
-      <c r="C137" s="4"/>
+      <c r="C137" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A138" s="9">
+      <c r="A138" s="9"/>
+      <c r="C138" s="4"/>
+      <c r="D138" s="8" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A139" s="9"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A140" s="9"/>
+      <c r="C140" s="4"/>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A141" s="9">
         <v>3</v>
       </c>
-      <c r="C138" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D138" s="8" t="s">
+      <c r="C141" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D141" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A142" s="9"/>
+      <c r="C142" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D142" s="8" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A139" s="9"/>
-      <c r="C139" s="6" t="s">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="11"/>
+      <c r="B143" s="8"/>
+      <c r="C143" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="D139" s="8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A140" s="11"/>
-      <c r="B140" s="8"/>
-      <c r="C140" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D140" s="8"/>
-    </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A141" s="9"/>
-      <c r="C141" s="4"/>
-    </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A142" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="B142" s="16"/>
-      <c r="C142" s="4"/>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="9">
-        <v>1</v>
-      </c>
-      <c r="C143" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="D143" s="8" t="s">
-        <v>150</v>
-      </c>
+      <c r="D143" s="8"/>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="9"/>
-      <c r="C144" s="6" t="s">
+      <c r="C144" s="4"/>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B145" s="23"/>
+      <c r="C145" s="4"/>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" s="9">
+        <v>1</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D146" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="9"/>
+      <c r="C147" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D147" s="8" t="s">
         <v>149</v>
-      </c>
-      <c r="D144" s="8" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A145" s="9"/>
-      <c r="C145" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D145" s="8"/>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A146" s="9"/>
-      <c r="C146" s="4"/>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A147" s="9">
-        <v>2</v>
-      </c>
-      <c r="C147" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="D147" s="8" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="9"/>
       <c r="C148" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D148" s="8" t="s">
-        <v>83</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="D148" s="8"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="9"/>
-      <c r="C149" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="D149" s="8" t="s">
-        <v>155</v>
-      </c>
+      <c r="C149" s="4"/>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A150" s="9"/>
-      <c r="C150" s="4"/>
+      <c r="A150" s="9">
+        <v>2</v>
+      </c>
+      <c r="C150" s="6" t="s">
+        <v>146</v>
+      </c>
       <c r="D150" s="8" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="9"/>
-      <c r="C151" s="4"/>
+      <c r="C151" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="D151" s="8" t="s">
-        <v>157</v>
+        <v>81</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="9"/>
-      <c r="C152" s="4"/>
+      <c r="C152" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D152" s="8" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" s="9">
+      <c r="A153" s="9"/>
+      <c r="C153" s="4"/>
+      <c r="D153" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" s="9"/>
+      <c r="C154" s="4"/>
+      <c r="D154" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" s="9"/>
+      <c r="C155" s="4"/>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156" s="9">
         <v>3</v>
       </c>
-      <c r="C153" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D153" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A154" s="11"/>
-      <c r="B154" s="8"/>
-      <c r="C154" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D154" s="8"/>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="11"/>
-      <c r="B155" s="8"/>
-      <c r="C155" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D155" s="8"/>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" s="9"/>
-      <c r="C156" s="4"/>
+      <c r="C156" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D156" s="8" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="9">
-        <v>4</v>
-      </c>
+      <c r="A157" s="11"/>
+      <c r="B157" s="8"/>
       <c r="C157" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D157" s="8" t="s">
-        <v>145</v>
-      </c>
+      <c r="D157" s="8"/>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" s="9"/>
+      <c r="A158" s="11"/>
+      <c r="B158" s="8"/>
       <c r="C158" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D158" s="8" t="s">
-        <v>147</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="D158" s="8"/>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="9"/>
-      <c r="C159" s="6" t="s">
+      <c r="C159" s="4"/>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160" s="9">
+        <v>4</v>
+      </c>
+      <c r="C160" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D160" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" s="9"/>
+      <c r="C161" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D161" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A162" s="9"/>
+      <c r="C162" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D162" s="8"/>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163" s="9"/>
+      <c r="C163" s="4"/>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A164" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B164" s="23"/>
+      <c r="C164" s="4"/>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165" s="9">
+        <v>1</v>
+      </c>
+      <c r="C165" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D165" s="8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A166" s="9"/>
+      <c r="C166" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="D159" s="8"/>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" s="9"/>
-      <c r="C160" s="4"/>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A161" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="B161" s="16"/>
-      <c r="C161" s="4"/>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A162" s="9">
-        <v>1</v>
-      </c>
-      <c r="C162" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D162" s="8" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A163" s="9"/>
-      <c r="C163" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D163" s="8" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A164" s="9"/>
-      <c r="C164" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D164" s="8" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" s="9"/>
-      <c r="C165" s="4"/>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A166" s="9">
-        <v>2</v>
-      </c>
-      <c r="C166" s="6" t="s">
-        <v>161</v>
-      </c>
       <c r="D166" s="8" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="9"/>
       <c r="C167" s="6" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="9"/>
-      <c r="C168" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D168" s="8" t="s">
+      <c r="C168" s="4"/>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169" s="9">
+        <v>2</v>
+      </c>
+      <c r="C169" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D169" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A170" s="9"/>
+      <c r="C170" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D170" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A171" s="9"/>
+      <c r="C171" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D171" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A173" s="2">
+        <v>3</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D173" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A174" s="8"/>
+      <c r="B174" s="8"/>
+      <c r="C174" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D174" s="8"/>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A175" s="8"/>
+      <c r="B175" s="8"/>
+      <c r="C175" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D175" s="8"/>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A177" s="2">
+        <v>4</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D177" s="8"/>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C178" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D178" s="8"/>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C179" s="3"/>
+      <c r="D179" s="8"/>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" s="2">
+        <v>5</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C182" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" s="2">
-        <v>3</v>
-      </c>
-      <c r="C170" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D170" s="8"/>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" s="8"/>
-      <c r="B171" s="8"/>
-      <c r="C171" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D171" s="8"/>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A172" s="8"/>
-      <c r="B172" s="8"/>
-      <c r="C172" s="3"/>
-      <c r="D172" s="8"/>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A174" s="2">
-        <v>4</v>
-      </c>
-      <c r="C174" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D174" s="8"/>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C175" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D175" s="8"/>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C176" s="3"/>
-      <c r="D176" s="8"/>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" s="2">
-        <v>5</v>
-      </c>
-      <c r="C178" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C179" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A142:B142"/>
-    <mergeCell ref="A161:B161"/>
-    <mergeCell ref="A23:B23"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="A105:B105"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
User Stories all functions
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89e05dc7f8bbc142/Documents/GitHub/Software-Engineering-Project-G1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A00329624\Documents\GitHub\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{98740330-EDCD-4F3B-BF22-E68E8C5CB1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C5930A-661F-4325-A644-1182943C4B14}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A75572F-76A8-4BE1-ACAE-4A6EE95B9735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="191">
   <si>
     <t>Number</t>
   </si>
@@ -548,12 +548,6 @@
     <t>Verify that when a delivery is not marked as successful, it is rescheduled to a later date</t>
   </si>
   <si>
-    <t>I want to read</t>
-  </si>
-  <si>
-    <t>I want to delete</t>
-  </si>
-  <si>
     <t>Verify that the customers address is printed to the screen</t>
   </si>
   <si>
@@ -578,7 +572,43 @@
     <t>so that my delivery people can know what deliveries need to be made on a given day</t>
   </si>
   <si>
-    <t>Verify that all orders on the order database are entered onto the delivery docket, including the order ID, order date, customer ID, customer address, customer name and order item</t>
+    <t>Verify that a valid(existing on the odrer database) order ID can be entered onto the delivery docket</t>
+  </si>
+  <si>
+    <t>Verify that if an invalid order ID is entered, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if a valid order ID is entered, all details contained under that order ID are added to the delivery docket</t>
+  </si>
+  <si>
+    <t>As a newsagent + delivery person</t>
+  </si>
+  <si>
+    <t>so that the drivers can bring a printed list of the orders they need to deliver</t>
+  </si>
+  <si>
+    <t>I want to read a delivery docket on a given day</t>
+  </si>
+  <si>
+    <t>Verify that all orders on a delivery docket for a given day are printed, one for each area.</t>
+  </si>
+  <si>
+    <t>Verify that if there are any areas with no deliveries, a docket is not printed</t>
+  </si>
+  <si>
+    <t>I want to delete a delivery docket</t>
+  </si>
+  <si>
+    <t>so that old delivery dockets are removed, to free up space</t>
+  </si>
+  <si>
+    <t>Verify that a docket can only be deleted if all deliveries on the docket were made successfully</t>
+  </si>
+  <si>
+    <t>Verify that if deliveries were not made successfully, those orders are transferred to a later delivery docket</t>
+  </si>
+  <si>
+    <t>Verify that the delivery docket is deleted from the system.</t>
   </si>
 </sst>
 </file>
@@ -718,6 +748,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -728,9 +761,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1067,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
-  <dimension ref="A1:J182"/>
+  <dimension ref="A1:J183"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
@@ -1079,10 +1109,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
+      <c r="B1" s="23"/>
       <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
@@ -1091,10 +1121,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="21"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -1653,7 +1683,7 @@
         <v>4</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -1666,7 +1696,7 @@
         <v>37</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -1680,7 +1710,7 @@
         <v>5</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -1691,7 +1721,7 @@
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
       <c r="D49" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -1868,7 +1898,7 @@
         <v>71</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -1878,7 +1908,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D64" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
@@ -1890,7 +1920,7 @@
       <c r="A65" s="9"/>
       <c r="C65" s="5"/>
       <c r="D65" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -1926,7 +1956,7 @@
       <c r="A68" s="9"/>
       <c r="C68" s="5"/>
       <c r="D68" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
@@ -1993,7 +2023,7 @@
       <c r="A73" s="9"/>
       <c r="C73" s="5"/>
       <c r="D73" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
@@ -2026,7 +2056,7 @@
       <c r="A76" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="B76" s="23"/>
+      <c r="B76" s="19"/>
       <c r="C76" s="5"/>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
@@ -2430,7 +2460,7 @@
       <c r="A108" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B108" s="23"/>
+      <c r="B108" s="19"/>
       <c r="C108" s="5"/>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
@@ -2831,7 +2861,7 @@
       <c r="A145" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="B145" s="23"/>
+      <c r="B145" s="19"/>
       <c r="C145" s="4"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -2978,7 +3008,7 @@
       <c r="A164" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B164" s="23"/>
+      <c r="B164" s="19"/>
       <c r="C164" s="4"/>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
@@ -3051,42 +3081,52 @@
         <v>146</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="8"/>
       <c r="B174" s="8"/>
       <c r="C174" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D174" s="8"/>
+        <v>176</v>
+      </c>
+      <c r="D174" s="8" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="8"/>
       <c r="B175" s="8"/>
       <c r="C175" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="D175" s="8"/>
+        <v>177</v>
+      </c>
+      <c r="D175" s="8" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>4</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D177" s="8"/>
+        <v>181</v>
+      </c>
+      <c r="D177" s="8" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C178" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D178" s="8"/>
+        <v>183</v>
+      </c>
+      <c r="D178" s="8" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C179" s="3"/>
+      <c r="C179" s="3" t="s">
+        <v>182</v>
+      </c>
       <c r="D179" s="8"/>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
@@ -3096,10 +3136,24 @@
       <c r="C181" s="2" t="s">
         <v>146</v>
       </c>
+      <c r="D181" s="2" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C182" s="2" t="s">
-        <v>171</v>
+        <v>186</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C183" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D183" s="2" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CRUD for most that were missing it
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A00329624\Documents\GitHub\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A75572F-76A8-4BE1-ACAE-4A6EE95B9735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE47721-A6F1-4072-8EE8-FA3FC3676FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="238">
   <si>
     <t>Number</t>
   </si>
@@ -101,45 +101,21 @@
     <t>Newsagent</t>
   </si>
   <si>
-    <t>Verify that a valid(3-50 characters) delivery person name can be entered</t>
-  </si>
-  <si>
-    <t>Verify that a valid(from 1 to the total number of areas) area code can be entered</t>
-  </si>
-  <si>
-    <t>Verify that a valid(only integers) delivery person phone number can be entered</t>
-  </si>
-  <si>
     <t>Verify that if any delivery person details entered are invalid, an error message is returned</t>
   </si>
   <si>
-    <t>Verify that if all entered values are valid, the delivery person and their details are put onto the database</t>
-  </si>
-  <si>
     <t>I want to delete a delivery person</t>
   </si>
   <si>
     <t>so that if one of my employees leaves, their details can be removed from the system</t>
   </si>
   <si>
-    <t>Verify that a delivery person can be selected for deletion via their area code, as only one delivery person can cover an area at a time</t>
-  </si>
-  <si>
-    <t>Verify that if an invalid(beyond the total number of areas) area code is entered, an error message is returned</t>
-  </si>
-  <si>
     <t>Verify that if the area code is valid, the user is promted if they are sure they want to delete this delivery person from the database</t>
   </si>
   <si>
-    <t>Verify that if the user selects yes, the delivery person is removed from the database</t>
-  </si>
-  <si>
     <t>Verify that if a valid customer ID is entered for deletion, the user is asked if they are sure they want to delete the customer</t>
   </si>
   <si>
-    <t>Verify that if the user selects yes, the customer is removed from the database</t>
-  </si>
-  <si>
     <t>Verify that if the user selects no, they are sent back to the system home page</t>
   </si>
   <si>
@@ -266,9 +242,6 @@
     <t>Verify that a valid(already present on the customer database) customer ID can be entered (Customer IDs would link back to all the customer details, including address)</t>
   </si>
   <si>
-    <t>Verify that if all entered values are valid, the entered order is put onto the order database</t>
-  </si>
-  <si>
     <t>I want to delete an order</t>
   </si>
   <si>
@@ -287,9 +260,6 @@
     <t>Verify that the user is asked if they are sure they want to delete this order</t>
   </si>
   <si>
-    <t>Verify that if the user selects yes, the order is removed from the database</t>
-  </si>
-  <si>
     <t>I want to update an order</t>
   </si>
   <si>
@@ -305,9 +275,6 @@
     <t>Verify that if either updated values are invalid, an error message is returned</t>
   </si>
   <si>
-    <t>Verify that after entering all details, if they are valid, the order is updated on the database while retaining its original order ID</t>
-  </si>
-  <si>
     <t>I want to read the order list</t>
   </si>
   <si>
@@ -347,15 +314,9 @@
     <t>I want to create a delivery area</t>
   </si>
   <si>
-    <t>Verify that a valid(greater than zero, not already existing area code) area code can be entered</t>
-  </si>
-  <si>
     <t>Verify that if the entered value is invalid, return an error message</t>
   </si>
   <si>
-    <t>Verify that if all entered values are valid, the customer and their details are put onto the database, attached to the entered area code</t>
-  </si>
-  <si>
     <t>I want to delete a delivery area</t>
   </si>
   <si>
@@ -365,9 +326,6 @@
     <t>Verify that a valid(existing area code) area code can be entered to select which area will be removed</t>
   </si>
   <si>
-    <t>Verify that if the entered value is valid, a new empty area is added to the area database</t>
-  </si>
-  <si>
     <t>Verify that if the entered code is valid, and if there are no customers in the area, the area is deleted</t>
   </si>
   <si>
@@ -389,9 +347,6 @@
     <t>Verify that if the entered value is invalid(less than or equal to 0, or not an integer), return an error message</t>
   </si>
   <si>
-    <t>Verify that if the entered value is valid, the area code is updated to the entered value</t>
-  </si>
-  <si>
     <t>I want to read a delivery area</t>
   </si>
   <si>
@@ -413,12 +368,6 @@
     <t>so that my business recieves the income it is owed for the service it provides</t>
   </si>
   <si>
-    <t>I want a bill for every customer to be automatically created at the start of each month</t>
-  </si>
-  <si>
-    <t>As a newsagent (Bill)</t>
-  </si>
-  <si>
     <t>I want to include the bill with the next delivery for a given customer</t>
   </si>
   <si>
@@ -449,24 +398,12 @@
     <t>Verify that if the bill is unpaid after two months, it is sent along with the next bill, alongside a solicitors letter</t>
   </si>
   <si>
-    <t>Verify that if the bill is unpaid after two months, the customer is deleted from the system</t>
-  </si>
-  <si>
-    <t>Verify that each customer ID recieves its own bill, detailing all of the previous months deliveries and their prices, as well as a total sum cost.</t>
-  </si>
-  <si>
     <t>As a newsagent (Publications)</t>
   </si>
   <si>
     <t>so that I know what publications are available for deliveries</t>
   </si>
   <si>
-    <t>I want to receive a notification when 5 or less of a publication are available</t>
-  </si>
-  <si>
-    <t>so that I know that it is time to set/reset stock</t>
-  </si>
-  <si>
     <t>Verify that the stock level of a publication goes down when it is delivered.</t>
   </si>
   <si>
@@ -494,9 +431,6 @@
     <t>so that I can set stock levels, or change the publications name</t>
   </si>
   <si>
-    <t>Verify that a valid(already on the database) publication name can be entered to select which publication to modify</t>
-  </si>
-  <si>
     <t>Verify that if the entered value is valid, the user is prompted to enter the new stock level</t>
   </si>
   <si>
@@ -509,9 +443,6 @@
     <t>Publications</t>
   </si>
   <si>
-    <t>Verify that when less than five of a publication are in stock, the user is notified: "Warning, 5 or less of [PUBLICATION] are present"</t>
-  </si>
-  <si>
     <t>so that I can ensure the stock count is identical between the system and in storage</t>
   </si>
   <si>
@@ -542,9 +473,6 @@
     <t>Verify that all areas are printed out, with the exception of any 'empty' areas (areas with no customers attached ot them</t>
   </si>
   <si>
-    <t>Verify that when a delivery is marked as successful, it is taken of the order databas</t>
-  </si>
-  <si>
     <t>Verify that when a delivery is not marked as successful, it is rescheduled to a later date</t>
   </si>
   <si>
@@ -554,9 +482,6 @@
     <t>Verify that a valid customer address can be entered</t>
   </si>
   <si>
-    <t>Verify that, if all entered values are valid, the Customers name, address and phone number are updated on the database</t>
-  </si>
-  <si>
     <t>Verify that a valid(1 or more characters) customer first name can be entered</t>
   </si>
   <si>
@@ -572,15 +497,9 @@
     <t>so that my delivery people can know what deliveries need to be made on a given day</t>
   </si>
   <si>
-    <t>Verify that a valid(existing on the odrer database) order ID can be entered onto the delivery docket</t>
-  </si>
-  <si>
     <t>Verify that if an invalid order ID is entered, an error message is returned</t>
   </si>
   <si>
-    <t>Verify that if a valid order ID is entered, all details contained under that order ID are added to the delivery docket</t>
-  </si>
-  <si>
     <t>As a newsagent + delivery person</t>
   </si>
   <si>
@@ -608,7 +527,229 @@
     <t>Verify that if deliveries were not made successfully, those orders are transferred to a later delivery docket</t>
   </si>
   <si>
-    <t>Verify that the delivery docket is deleted from the system.</t>
+    <t>I want to read the bill</t>
+  </si>
+  <si>
+    <t>so that I can charge my customers for the service I provide</t>
+  </si>
+  <si>
+    <t>Verify that the bill includes the Customer ID it corresponds to</t>
+  </si>
+  <si>
+    <t>Verify that the bill includes all orders made under that customer ID over the previous month</t>
+  </si>
+  <si>
+    <t>Verify that the bill includes the sum total of costs from all orders over the previous month</t>
+  </si>
+  <si>
+    <t>I want to update the bill</t>
+  </si>
+  <si>
+    <t>so that new orders can be added to a pre-existing bill</t>
+  </si>
+  <si>
+    <t>Verify that a valid(exists on the order database) can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if a valid order ID Is entered, the order is appended to the end of the bill</t>
+  </si>
+  <si>
+    <t>Verify that the cost of the new order is added to the sum total of the bill</t>
+  </si>
+  <si>
+    <t>I want to delete a bill</t>
+  </si>
+  <si>
+    <t>so that</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the customer is created</t>
+  </si>
+  <si>
+    <t>Verify that, if all entered values are valid, the Customers name, address and phone number are updated</t>
+  </si>
+  <si>
+    <t>Verify that if the user selects yes, the delivery person is removed</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the delivery person is created</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the order is created</t>
+  </si>
+  <si>
+    <t>Verify that if the user selects yes, the order is removed</t>
+  </si>
+  <si>
+    <t>Verify that after entering all details, if they are valid, the order is updated</t>
+  </si>
+  <si>
+    <t>Verify that a valid(2 or more characters) area code can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if the bill is unpaid after two months, the customer is deleted</t>
+  </si>
+  <si>
+    <t>Verify that when a delivery is marked as successful, it is removed</t>
+  </si>
+  <si>
+    <t>Verify that the delivery docket is deleted</t>
+  </si>
+  <si>
+    <t>I want to create a publication</t>
+  </si>
+  <si>
+    <t>so that I can fulfill the needs/wants of my customers</t>
+  </si>
+  <si>
+    <t>Verify that a valid publication name can be added(more than 3 characters)</t>
+  </si>
+  <si>
+    <t>Verify that a valid publication stock can be added(greater than 0)</t>
+  </si>
+  <si>
+    <t>Verify that if an invalid name is entered, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if an invalid stock is entered, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if both entered values are valid, the publication is created.</t>
+  </si>
+  <si>
+    <t>I want to delete a publication</t>
+  </si>
+  <si>
+    <t>so that I can remove any publications I no longer sell</t>
+  </si>
+  <si>
+    <t>Verify that an existing publication name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if the entered name does not exist, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if the entered name does exist, the publication is deleted.</t>
+  </si>
+  <si>
+    <t>Verify that if a valid order ID is entered, a delivery docket is created with the entered order ID included</t>
+  </si>
+  <si>
+    <t>Verify that a valid customer ID can be entered (existing)</t>
+  </si>
+  <si>
+    <t>Verify that if the entered value is valid, the bill is deleted</t>
+  </si>
+  <si>
+    <t>Verify that if the entered value is valid, the area is updated</t>
+  </si>
+  <si>
+    <t>I want to create a bill</t>
+  </si>
+  <si>
+    <t>Verify that an existing customer ID can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid date can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if the entered customer ID does not exist, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that an existing order ID(s) can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if the entered order ID does not exist, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if an invalid date is entered, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid/existing, a bill is created</t>
+  </si>
+  <si>
+    <t>Verify that if a publication has less than 5 in stock, a message warning the user is returned "Warning: Less than 5 of [publication] remaining"</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) publication name can be entered to select which publication to modify</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing order) order ID can be entered onto the delivery docket</t>
+  </si>
+  <si>
+    <t>I want to read a delivery person</t>
+  </si>
+  <si>
+    <t>so that I can view the information of a delivery person</t>
+  </si>
+  <si>
+    <t>Verify that a valid(more than 2 characters, existing area) area code can be entered</t>
+  </si>
+  <si>
+    <t>Verify that the delivery person area code is returned</t>
+  </si>
+  <si>
+    <t>Verify that the delivery person name is returned</t>
+  </si>
+  <si>
+    <t>Verify that the deliver person phone number is returned</t>
+  </si>
+  <si>
+    <t>so that I can edit the details of my employees</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) delivery person name can be entered to select the deliver person</t>
+  </si>
+  <si>
+    <t>Verify that a valid(3 or more characters) delivery person first name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(3 or more characters) delivery person last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(10 numbers) delivery person phone number can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) delivery person last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if an invalid value is entered, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that a valid(more 2 characters) delivery person first name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(more 2 characters) delivery person last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(10 numbers) phone number can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(2 or more characters, existing area code) area code can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the delivery person is updated</t>
+  </si>
+  <si>
+    <t>Verify that if any entered values are invalid, an error message is returned</t>
+  </si>
+  <si>
+    <t>As a Newsagent (Bill)</t>
+  </si>
+  <si>
+    <t>Verify that if the user selects yes, the customer is  deleted</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) customer ID can be entered</t>
+  </si>
+  <si>
+    <t>if the entered value is invalid, return an error message</t>
+  </si>
+  <si>
+    <t>Verify that both entered values are valid, a new area is created</t>
+  </si>
+  <si>
+    <t>I want to update a delivery person</t>
   </si>
 </sst>
 </file>
@@ -1097,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
-  <dimension ref="A1:J183"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
@@ -1135,7 +1276,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>221</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1145,30 +1286,15 @@
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="C4" s="5" t="s">
-        <v>36</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+        <v>222</v>
+      </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="C5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1176,9 +1302,11 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
-      <c r="C6" s="5"/>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>215</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1189,9 +1317,11 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
-      <c r="C7" s="5"/>
+      <c r="C7" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="D7" s="2" t="s">
-        <v>25</v>
+        <v>223</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1203,6 +1333,9 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="C8" s="5"/>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -1211,14 +1344,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
-        <v>2</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A9" s="9"/>
+      <c r="C9" s="5"/>
       <c r="D9" s="2" t="s">
-        <v>28</v>
+        <v>178</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1229,12 +1358,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
-      <c r="C10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="C10" s="5"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
@@ -1243,12 +1367,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
+      <c r="A11" s="9">
+        <v>2</v>
+      </c>
       <c r="C11" s="5" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>224</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1259,9 +1385,11 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
-      <c r="C12" s="5"/>
+      <c r="C12" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="D12" s="2" t="s">
-        <v>31</v>
+        <v>225</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -1272,9 +1400,11 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
-      <c r="C13" s="5"/>
+      <c r="C13" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="D13" s="2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -1285,17 +1415,18 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="9">
-        <v>3</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A15" s="9"/>
+      <c r="C15" s="5"/>
       <c r="D15" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -1305,25 +1436,20 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
-      <c r="C16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="C16" s="4"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
+      <c r="A17" s="9">
+        <v>3</v>
+      </c>
       <c r="C17" s="5" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1332,6 +1458,13 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="C18" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -1340,7 +1473,12 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
-      <c r="C19" s="5"/>
+      <c r="C19" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -1348,15 +1486,6 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="9">
-        <v>4</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -1365,9 +1494,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
-      <c r="C21" s="5" t="s">
-        <v>48</v>
-      </c>
+      <c r="C21" s="5"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
@@ -1375,9 +1502,14 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
+      <c r="A22" s="9">
+        <v>4</v>
+      </c>
       <c r="C22" s="5" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -1387,7 +1519,9 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="9"/>
-      <c r="C23" s="5"/>
+      <c r="C23" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -1395,11 +1529,10 @@
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="5"/>
+      <c r="A24" s="9"/>
+      <c r="C24" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -1407,15 +1540,8 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="9">
-        <v>1</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="A25" s="9"/>
+      <c r="C25" s="5"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -1423,12 +1549,14 @@
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="9"/>
-      <c r="C26" s="5" t="s">
-        <v>38</v>
+      <c r="A26" s="2">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>41</v>
+        <v>220</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1437,12 +1565,11 @@
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="9"/>
-      <c r="C27" s="5" t="s">
-        <v>45</v>
+      <c r="C27" s="2" t="s">
+        <v>213</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -1451,8 +1578,12 @@
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="9"/>
-      <c r="C28" s="5"/>
+      <c r="C28" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>217</v>
+      </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
@@ -1460,14 +1591,8 @@
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="9">
-        <v>2</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="D29" s="2" t="s">
-        <v>47</v>
+        <v>216</v>
       </c>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -1475,13 +1600,9 @@
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
-      <c r="C30" s="5" t="s">
-        <v>55</v>
-      </c>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D30" s="2" t="s">
-        <v>53</v>
+        <v>218</v>
       </c>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -1490,13 +1611,6 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
-      <c r="C31" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
@@ -1504,10 +1618,14 @@
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
-      <c r="C32" s="5"/>
+      <c r="A32" s="2">
+        <v>6</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="D32" s="2" t="s">
-        <v>51</v>
+        <v>220</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -1516,8 +1634,12 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="9"/>
-      <c r="C33" s="5"/>
+      <c r="C33" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
@@ -1525,14 +1647,11 @@
       <c r="I33" s="1"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="9">
-        <v>3</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>44</v>
+      <c r="C34" s="2" t="s">
+        <v>219</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>58</v>
+        <v>226</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -1541,12 +1660,8 @@
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
-      <c r="C35" s="5" t="s">
-        <v>56</v>
-      </c>
       <c r="D35" s="2" t="s">
-        <v>59</v>
+        <v>227</v>
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -1555,9 +1670,8 @@
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="9"/>
-      <c r="C36" s="5" t="s">
-        <v>57</v>
+      <c r="D36" s="2" t="s">
+        <v>229</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -1566,8 +1680,9 @@
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="9"/>
-      <c r="C37" s="5"/>
+      <c r="D37" s="2" t="s">
+        <v>228</v>
+      </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -1575,14 +1690,8 @@
       <c r="I37" s="1"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="9">
-        <v>4</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>44</v>
-      </c>
       <c r="D38" s="2" t="s">
-        <v>63</v>
+        <v>231</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -1591,12 +1700,8 @@
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
-      <c r="C39" s="5" t="s">
-        <v>61</v>
-      </c>
       <c r="D39" s="2" t="s">
-        <v>64</v>
+        <v>230</v>
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -1605,13 +1710,6 @@
       <c r="I39" s="1"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="9"/>
-      <c r="C40" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
@@ -1619,11 +1717,11 @@
       <c r="I40" s="1"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="9"/>
+      <c r="A41" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41" s="16"/>
       <c r="C41" s="5"/>
-      <c r="D41" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
@@ -1631,10 +1729,14 @@
       <c r="I41" s="1"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="9"/>
-      <c r="C42" s="5"/>
+      <c r="A42" s="9">
+        <v>1</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="D42" s="2" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -1644,9 +1746,11 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
-      <c r="C43" s="5"/>
+      <c r="C43" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="D43" s="2" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -1656,7 +1760,12 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
-      <c r="C44" s="5"/>
+      <c r="C44" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
@@ -1664,10 +1773,7 @@
       <c r="I44" s="1"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A45" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="B45" s="18"/>
+      <c r="A45" s="9"/>
       <c r="C45" s="5"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -1677,13 +1783,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
-        <v>1</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>173</v>
+        <v>2</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -1691,12 +1797,13 @@
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C47" s="6" t="s">
-        <v>37</v>
+    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="9"/>
+      <c r="C47" s="5" t="s">
+        <v>47</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -1706,11 +1813,11 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
-      <c r="C48" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>171</v>
+      <c r="C48" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -1720,8 +1827,9 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-      <c r="D49" s="8" t="s">
-        <v>175</v>
+      <c r="C49" s="5"/>
+      <c r="D49" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -1732,9 +1840,6 @@
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
       <c r="C50" s="5"/>
-      <c r="D50" s="8" t="s">
-        <v>60</v>
-      </c>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
@@ -1742,10 +1847,14 @@
       <c r="I50" s="1"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="9"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="8" t="s">
-        <v>13</v>
+      <c r="A51" s="9">
+        <v>3</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -1755,9 +1864,11 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="8" t="s">
-        <v>105</v>
+      <c r="C52" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -1767,9 +1878,8 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="8" t="s">
-        <v>10</v>
+      <c r="C53" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -1779,6 +1889,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
+      <c r="C54" s="5"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
@@ -1787,13 +1898,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="9">
-        <v>2</v>
-      </c>
-      <c r="C55" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D55" s="8" t="s">
-        <v>11</v>
+      <c r="C55" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -1803,11 +1914,11 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
-      <c r="C56" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>12</v>
+      <c r="C56" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -1817,11 +1928,11 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="9"/>
-      <c r="C57" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>32</v>
+      <c r="C57" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -1832,8 +1943,8 @@
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
       <c r="C58" s="5"/>
-      <c r="D58" s="8" t="s">
-        <v>33</v>
+      <c r="D58" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
@@ -1844,8 +1955,8 @@
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="9"/>
       <c r="C59" s="5"/>
-      <c r="D59" s="8" t="s">
-        <v>34</v>
+      <c r="D59" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
@@ -1856,6 +1967,9 @@
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="9"/>
       <c r="C60" s="5"/>
+      <c r="D60" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
@@ -1863,15 +1977,8 @@
       <c r="I60" s="1"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="9">
-        <v>3</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="A61" s="9"/>
+      <c r="C61" s="5"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
@@ -1879,13 +1986,11 @@
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="9"/>
-      <c r="C62" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>12</v>
-      </c>
+      <c r="A62" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B62" s="18"/>
+      <c r="C62" s="5"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
@@ -1893,12 +1998,14 @@
       <c r="I62" s="1"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="9"/>
+      <c r="A63" s="9">
+        <v>1</v>
+      </c>
       <c r="C63" s="6" t="s">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -1907,8 +2014,11 @@
       <c r="I63" s="1"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C64" s="6" t="s">
+        <v>29</v>
+      </c>
       <c r="D64" s="2" t="s">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
@@ -1918,9 +2028,11 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="9"/>
-      <c r="C65" s="5"/>
+      <c r="C65" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="D65" s="8" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
@@ -1930,9 +2042,8 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="9"/>
-      <c r="C66" s="5"/>
       <c r="D66" s="8" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
@@ -1944,7 +2055,7 @@
       <c r="A67" s="9"/>
       <c r="C67" s="5"/>
       <c r="D67" s="8" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
@@ -1956,7 +2067,7 @@
       <c r="A68" s="9"/>
       <c r="C68" s="5"/>
       <c r="D68" s="8" t="s">
-        <v>172</v>
+        <v>13</v>
       </c>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
@@ -1967,6 +2078,9 @@
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="9"/>
       <c r="C69" s="5"/>
+      <c r="D69" s="8" t="s">
+        <v>175</v>
+      </c>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
@@ -1974,14 +2088,10 @@
       <c r="I69" s="1"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A70" s="9">
-        <v>4</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>14</v>
+      <c r="A70" s="9"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
@@ -1990,14 +2100,7 @@
       <c r="I70" s="1"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A71" s="10"/>
-      <c r="B71" s="7"/>
-      <c r="C71" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="A71" s="9"/>
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
@@ -2005,13 +2108,14 @@
       <c r="I71" s="1"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A72" s="10"/>
-      <c r="B72" s="7"/>
+      <c r="A72" s="9">
+        <v>2</v>
+      </c>
       <c r="C72" s="6" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
@@ -2021,9 +2125,11 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="9"/>
-      <c r="C73" s="5"/>
+      <c r="C73" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="D73" s="8" t="s">
-        <v>170</v>
+        <v>12</v>
       </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
@@ -2033,9 +2139,11 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="9"/>
-      <c r="C74" s="5"/>
+      <c r="C74" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="D74" s="8" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
@@ -2046,6 +2154,9 @@
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="9"/>
       <c r="C75" s="5"/>
+      <c r="D75" s="8" t="s">
+        <v>233</v>
+      </c>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="G75" s="1"/>
@@ -2053,11 +2164,11 @@
       <c r="I75" s="1"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="B76" s="19"/>
+      <c r="A76" s="9"/>
       <c r="C76" s="5"/>
+      <c r="D76" s="8" t="s">
+        <v>26</v>
+      </c>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
@@ -2065,15 +2176,8 @@
       <c r="I76" s="1"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="9">
-        <v>1</v>
-      </c>
-      <c r="C77" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>72</v>
-      </c>
+      <c r="A77" s="9"/>
+      <c r="C77" s="5"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
@@ -2081,12 +2185,14 @@
       <c r="I77" s="1"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="9"/>
-      <c r="C78" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>75</v>
+      <c r="A78" s="9">
+        <v>3</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
@@ -2096,11 +2202,11 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
-      <c r="C79" s="5" t="s">
-        <v>5</v>
+      <c r="C79" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="1"/>
@@ -2110,9 +2216,11 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
-      <c r="C80" s="5"/>
+      <c r="C80" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="D80" s="8" t="s">
-        <v>74</v>
+        <v>148</v>
       </c>
       <c r="E80" s="1"/>
       <c r="F80" s="1"/>
@@ -2121,10 +2229,8 @@
       <c r="I80" s="1"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="9"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="8" t="s">
-        <v>76</v>
+      <c r="D81" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="E81" s="1"/>
       <c r="F81" s="1"/>
@@ -2136,7 +2242,7 @@
       <c r="A82" s="9"/>
       <c r="C82" s="5"/>
       <c r="D82" s="8" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="E82" s="1"/>
       <c r="F82" s="1"/>
@@ -2147,6 +2253,9 @@
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
       <c r="C83" s="5"/>
+      <c r="D83" s="8" t="s">
+        <v>6</v>
+      </c>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
@@ -2154,14 +2263,10 @@
       <c r="I83" s="1"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="9">
-        <v>2</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A84" s="9"/>
+      <c r="C84" s="5"/>
       <c r="D84" s="8" t="s">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
@@ -2171,11 +2276,9 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
-      <c r="C85" s="5" t="s">
-        <v>77</v>
-      </c>
+      <c r="C85" s="5"/>
       <c r="D85" s="8" t="s">
-        <v>81</v>
+        <v>176</v>
       </c>
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
@@ -2185,12 +2288,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
-      <c r="C86" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>82</v>
-      </c>
+      <c r="C86" s="5"/>
       <c r="E86" s="1"/>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
@@ -2198,10 +2296,14 @@
       <c r="I86" s="1"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="9"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="8" t="s">
-        <v>83</v>
+      <c r="A87" s="9">
+        <v>4</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="E87" s="1"/>
       <c r="F87" s="1"/>
@@ -2210,10 +2312,13 @@
       <c r="I87" s="1"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88" s="9"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="8" t="s">
-        <v>34</v>
+      <c r="A88" s="10"/>
+      <c r="B88" s="7"/>
+      <c r="C88" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
@@ -2222,8 +2327,14 @@
       <c r="I88" s="1"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" s="9"/>
-      <c r="C89" s="5"/>
+      <c r="A89" s="10"/>
+      <c r="B89" s="7"/>
+      <c r="C89" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>17</v>
+      </c>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
@@ -2231,14 +2342,10 @@
       <c r="I89" s="1"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="9">
-        <v>3</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A90" s="9"/>
+      <c r="C90" s="5"/>
       <c r="D90" s="8" t="s">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
@@ -2248,11 +2355,9 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
-      <c r="C91" s="5" t="s">
-        <v>84</v>
-      </c>
+      <c r="C91" s="5"/>
       <c r="D91" s="8" t="s">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
@@ -2262,12 +2367,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
-      <c r="C92" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D92" s="8" t="s">
-        <v>82</v>
-      </c>
+      <c r="C92" s="5"/>
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
       <c r="G92" s="1"/>
@@ -2275,11 +2375,11 @@
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="9"/>
+      <c r="A93" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B93" s="19"/>
       <c r="C93" s="5"/>
-      <c r="D93" s="8" t="s">
-        <v>34</v>
-      </c>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
@@ -2287,10 +2387,14 @@
       <c r="I93" s="1"/>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" s="9"/>
-      <c r="C94" s="5"/>
+      <c r="A94" s="9">
+        <v>1</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D94" s="8" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
@@ -2300,9 +2404,11 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
-      <c r="C95" s="5"/>
+      <c r="C95" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="D95" s="8" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="E95" s="1"/>
       <c r="F95" s="1"/>
@@ -2312,9 +2418,11 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="9"/>
-      <c r="C96" s="5"/>
+      <c r="C96" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="D96" s="8" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
@@ -2326,7 +2434,7 @@
       <c r="A97" s="9"/>
       <c r="C97" s="5"/>
       <c r="D97" s="8" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
@@ -2337,6 +2445,9 @@
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
       <c r="C98" s="5"/>
+      <c r="D98" s="8" t="s">
+        <v>179</v>
+      </c>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
       <c r="G98" s="1"/>
@@ -2344,14 +2455,10 @@
       <c r="I98" s="1"/>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A99" s="9">
-        <v>4</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A99" s="9"/>
+      <c r="C99" s="5"/>
       <c r="D99" s="8" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E99" s="1"/>
       <c r="F99" s="1"/>
@@ -2361,12 +2468,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="9"/>
-      <c r="C100" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D100" s="8" t="s">
-        <v>93</v>
-      </c>
+      <c r="C100" s="5"/>
       <c r="E100" s="1"/>
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
@@ -2374,12 +2476,14 @@
       <c r="I100" s="1"/>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A101" s="9"/>
+      <c r="A101" s="9">
+        <v>2</v>
+      </c>
       <c r="C101" s="5" t="s">
-        <v>91</v>
+        <v>4</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="E101" s="1"/>
       <c r="F101" s="1"/>
@@ -2389,9 +2493,11 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="9"/>
-      <c r="C102" s="5"/>
+      <c r="C102" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="D102" s="8" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="E102" s="1"/>
       <c r="F102" s="1"/>
@@ -2401,9 +2507,11 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="9"/>
-      <c r="C103" s="5"/>
-      <c r="D103" s="2" t="s">
-        <v>96</v>
+      <c r="C103" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D103" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1"/>
@@ -2414,8 +2522,8 @@
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="9"/>
       <c r="C104" s="5"/>
-      <c r="D104" s="2" t="s">
-        <v>97</v>
+      <c r="D104" s="8" t="s">
+        <v>180</v>
       </c>
       <c r="E104" s="1"/>
       <c r="F104" s="1"/>
@@ -2427,7 +2535,7 @@
       <c r="A105" s="9"/>
       <c r="C105" s="5"/>
       <c r="D105" s="8" t="s">
-        <v>98</v>
+        <v>26</v>
       </c>
       <c r="E105" s="1"/>
       <c r="F105" s="1"/>
@@ -2438,9 +2546,6 @@
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="9"/>
       <c r="C106" s="5"/>
-      <c r="D106" s="8" t="s">
-        <v>99</v>
-      </c>
       <c r="E106" s="1"/>
       <c r="F106" s="1"/>
       <c r="G106" s="1"/>
@@ -2448,8 +2553,15 @@
       <c r="I106" s="1"/>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A107" s="9"/>
-      <c r="C107" s="5"/>
+      <c r="A107" s="9">
+        <v>3</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D107" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
@@ -2457,11 +2569,13 @@
       <c r="I107" s="1"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A108" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="B108" s="19"/>
-      <c r="C108" s="5"/>
+      <c r="A108" s="9"/>
+      <c r="C108" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
@@ -2469,14 +2583,12 @@
       <c r="I108" s="1"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A109" s="9">
-        <v>1</v>
-      </c>
+      <c r="A109" s="9"/>
       <c r="C109" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>103</v>
+        <v>75</v>
+      </c>
+      <c r="D109" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
@@ -2486,11 +2598,9 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="9"/>
-      <c r="C110" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>104</v>
+      <c r="C110" s="5"/>
+      <c r="D110" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
@@ -2500,11 +2610,9 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="9"/>
-      <c r="C111" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>109</v>
+      <c r="C111" s="5"/>
+      <c r="D111" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="E111" s="1"/>
       <c r="F111" s="1"/>
@@ -2515,6 +2623,9 @@
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="9"/>
       <c r="C112" s="5"/>
+      <c r="D112" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
       <c r="G112" s="1"/>
@@ -2522,14 +2633,10 @@
       <c r="I112" s="1"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="9">
-        <v>2</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>108</v>
+      <c r="A113" s="9"/>
+      <c r="C113" s="5"/>
+      <c r="D113" s="8" t="s">
+        <v>78</v>
       </c>
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
@@ -2539,11 +2646,9 @@
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="9"/>
-      <c r="C114" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>81</v>
+      <c r="C114" s="5"/>
+      <c r="D114" s="8" t="s">
+        <v>181</v>
       </c>
       <c r="E114" s="1"/>
       <c r="F114" s="1"/>
@@ -2553,12 +2658,7 @@
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="9"/>
-      <c r="C115" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D115" s="14" t="s">
-        <v>114</v>
-      </c>
+      <c r="C115" s="5"/>
       <c r="E115" s="1"/>
       <c r="F115" s="1"/>
       <c r="G115" s="1"/>
@@ -2566,10 +2666,14 @@
       <c r="I115" s="1"/>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A116" s="9"/>
-      <c r="C116" s="5"/>
-      <c r="D116" s="2" t="s">
-        <v>110</v>
+      <c r="A116" s="9">
+        <v>4</v>
+      </c>
+      <c r="C116" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D116" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
@@ -2579,7 +2683,12 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="9"/>
-      <c r="C117" s="5"/>
+      <c r="C117" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D117" s="8" t="s">
+        <v>82</v>
+      </c>
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
@@ -2587,14 +2696,12 @@
       <c r="I117" s="1"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" s="9">
-        <v>3</v>
-      </c>
+      <c r="A118" s="9"/>
       <c r="C118" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>113</v>
+        <v>80</v>
+      </c>
+      <c r="D118" s="8" t="s">
+        <v>83</v>
       </c>
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
@@ -2604,11 +2711,9 @@
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="9"/>
-      <c r="C119" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>81</v>
+      <c r="C119" s="5"/>
+      <c r="D119" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
@@ -2618,11 +2723,9 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="9"/>
-      <c r="C120" s="5" t="s">
-        <v>112</v>
-      </c>
+      <c r="C120" s="5"/>
       <c r="D120" s="2" t="s">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
@@ -2634,7 +2737,7 @@
       <c r="A121" s="9"/>
       <c r="C121" s="5"/>
       <c r="D121" s="2" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
@@ -2645,8 +2748,8 @@
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="9"/>
       <c r="C122" s="5"/>
-      <c r="D122" s="2" t="s">
-        <v>116</v>
+      <c r="D122" s="8" t="s">
+        <v>87</v>
       </c>
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
@@ -2657,8 +2760,8 @@
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="9"/>
       <c r="C123" s="5"/>
-      <c r="D123" s="2" t="s">
-        <v>117</v>
+      <c r="D123" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
@@ -2676,15 +2779,11 @@
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="9">
-        <v>4</v>
-      </c>
-      <c r="C125" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>120</v>
-      </c>
+      <c r="A125" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B125" s="19"/>
+      <c r="C125" s="5"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
@@ -2692,12 +2791,14 @@
       <c r="I125" s="1"/>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A126" s="9"/>
+      <c r="A126" s="9">
+        <v>1</v>
+      </c>
       <c r="C126" s="5" t="s">
-        <v>118</v>
+        <v>4</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>81</v>
+        <v>182</v>
       </c>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
@@ -2708,10 +2809,10 @@
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="9"/>
       <c r="C127" s="5" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
@@ -2721,9 +2822,11 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="9"/>
-      <c r="C128" s="5"/>
+      <c r="C128" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="D128" s="2" t="s">
-        <v>122</v>
+        <v>234</v>
       </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
@@ -2734,6 +2837,9 @@
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="9"/>
       <c r="C129" s="5"/>
+      <c r="D129" s="2" t="s">
+        <v>235</v>
+      </c>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
@@ -2741,10 +2847,9 @@
       <c r="I129" s="1"/>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A130" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C130" s="5"/>
+      <c r="D130" s="2" t="s">
+        <v>236</v>
+      </c>
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
@@ -2752,408 +2857,705 @@
       <c r="I130" s="1"/>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A131" s="9">
-        <v>1</v>
-      </c>
-      <c r="C131" s="5" t="s">
+      <c r="E131" s="1"/>
+      <c r="F131" s="1"/>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A132" s="9">
+        <v>2</v>
+      </c>
+      <c r="C132" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D131" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A132" s="9"/>
-      <c r="C132" s="5" t="s">
-        <v>125</v>
-      </c>
+      <c r="D132" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E132" s="1"/>
+      <c r="F132" s="1"/>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="9"/>
       <c r="C133" s="5" t="s">
-        <v>124</v>
+        <v>93</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="9"/>
-      <c r="C134" s="4"/>
+      <c r="C134" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D134" s="14" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A135" s="9">
-        <v>2</v>
-      </c>
-      <c r="C135" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D135" s="8" t="s">
-        <v>134</v>
+      <c r="A135" s="9"/>
+      <c r="C135" s="5"/>
+      <c r="D135" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="9"/>
-      <c r="C136" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D136" s="8" t="s">
-        <v>128</v>
-      </c>
+      <c r="C136" s="5"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A137" s="9"/>
-      <c r="C137" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D137" s="8" t="s">
-        <v>135</v>
+      <c r="A137" s="9">
+        <v>3</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="9"/>
-      <c r="C138" s="4"/>
-      <c r="D138" s="8" t="s">
-        <v>136</v>
+      <c r="C138" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="9"/>
-      <c r="C139" s="4"/>
-      <c r="D139" s="8" t="s">
-        <v>137</v>
+      <c r="C139" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="9"/>
-      <c r="C140" s="4"/>
+      <c r="C140" s="5"/>
+      <c r="D140" s="2" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A141" s="9">
-        <v>3</v>
-      </c>
-      <c r="C141" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D141" s="8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="142" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A141" s="9"/>
+      <c r="C141" s="5"/>
+      <c r="D141" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="9"/>
-      <c r="C142" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D142" s="8" t="s">
-        <v>132</v>
+      <c r="C142" s="5"/>
+      <c r="D142" s="2" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A143" s="11"/>
-      <c r="B143" s="8"/>
-      <c r="C143" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D143" s="8"/>
+      <c r="A143" s="9"/>
+      <c r="C143" s="5"/>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A144" s="9"/>
-      <c r="C144" s="4"/>
+      <c r="A144" s="9">
+        <v>4</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A145" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="B145" s="19"/>
-      <c r="C145" s="4"/>
+      <c r="A145" s="9"/>
+      <c r="C145" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A146" s="9">
-        <v>1</v>
-      </c>
-      <c r="C146" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D146" s="8" t="s">
-        <v>148</v>
+      <c r="A146" s="9"/>
+      <c r="C146" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="9"/>
-      <c r="C147" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="D147" s="8" t="s">
-        <v>149</v>
+      <c r="C147" s="5"/>
+      <c r="D147" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="9"/>
-      <c r="C148" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D148" s="8"/>
+      <c r="C148" s="5"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="9"/>
-      <c r="C149" s="4"/>
+      <c r="A149" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C149" s="5"/>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="9">
-        <v>2</v>
-      </c>
-      <c r="C150" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D150" s="8" t="s">
-        <v>152</v>
+        <v>1</v>
+      </c>
+      <c r="C150" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="9"/>
-      <c r="C151" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="D151" s="8" t="s">
-        <v>81</v>
+      <c r="C151" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="9"/>
-      <c r="C152" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="D152" s="8" t="s">
-        <v>153</v>
+      <c r="C152" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="9"/>
       <c r="C153" s="4"/>
-      <c r="D153" s="8" t="s">
-        <v>154</v>
+      <c r="D153" s="2" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A154" s="9"/>
-      <c r="C154" s="4"/>
-      <c r="D154" s="8" t="s">
-        <v>155</v>
+      <c r="D154" s="2" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="9"/>
-      <c r="C155" s="4"/>
+      <c r="D155" s="2" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" s="9">
-        <v>3</v>
-      </c>
-      <c r="C156" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="D156" s="8" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="11"/>
-      <c r="B157" s="8"/>
-      <c r="C157" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D157" s="8"/>
+      <c r="D156" s="2" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" s="11"/>
-      <c r="B158" s="8"/>
+      <c r="A158" s="9">
+        <v>2</v>
+      </c>
       <c r="C158" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D158" s="8"/>
+        <v>232</v>
+      </c>
+      <c r="D158" s="8" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="9"/>
-      <c r="C159" s="4"/>
+      <c r="C159" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D159" s="8" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A160" s="9">
-        <v>4</v>
-      </c>
+      <c r="A160" s="9"/>
       <c r="C160" s="6" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="D160" s="8" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="9"/>
-      <c r="C161" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="C161" s="4"/>
       <c r="D161" s="8" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="9"/>
-      <c r="C162" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="D162" s="8"/>
+      <c r="C162" s="4"/>
+      <c r="D162" s="8" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="9"/>
       <c r="C163" s="4"/>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A164" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="B164" s="19"/>
-      <c r="C164" s="4"/>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" s="9">
-        <v>1</v>
-      </c>
+      <c r="A164" s="9">
+        <v>3</v>
+      </c>
+      <c r="C164" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D164" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A165" s="9"/>
       <c r="C165" s="6" t="s">
-        <v>159</v>
+        <v>114</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A166" s="9"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A166" s="11"/>
+      <c r="B166" s="8"/>
       <c r="C166" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D166" s="8" t="s">
-        <v>166</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="D166" s="8"/>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="9"/>
-      <c r="C167" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D167" s="8" t="s">
+      <c r="C167" s="4"/>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A168" s="2">
+        <v>4</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C169" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C170" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D170" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A168" s="9"/>
-      <c r="C168" s="4"/>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A169" s="9">
-        <v>2</v>
-      </c>
-      <c r="C169" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D169" s="8" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A170" s="9"/>
-      <c r="C170" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="D170" s="8" t="s">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A172" s="2">
+        <v>5</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C173" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" s="9"/>
-      <c r="C171" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D171" s="8" t="s">
+      <c r="D173" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C174" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A173" s="2">
-        <v>3</v>
-      </c>
-      <c r="C173" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D173" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A174" s="8"/>
-      <c r="B174" s="8"/>
-      <c r="C174" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D174" s="8" t="s">
-        <v>179</v>
+      <c r="D174" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A175" s="8"/>
-      <c r="B175" s="8"/>
-      <c r="C175" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="D175" s="8" t="s">
-        <v>180</v>
+      <c r="D175" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
+        <v>6</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C178" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C179" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="B180" s="19"/>
+      <c r="C180" s="4"/>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181" s="9">
+        <v>1</v>
+      </c>
+      <c r="C181" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D181" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182" s="9"/>
+      <c r="C182" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D182" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183" s="9"/>
+      <c r="C183" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D183" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184" s="9"/>
+      <c r="C184" s="4"/>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185" s="9">
+        <v>2</v>
+      </c>
+      <c r="C185" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D185" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A186" s="9"/>
+      <c r="C186" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D186" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187" s="9"/>
+      <c r="C187" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D187" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188" s="9"/>
+      <c r="C188" s="4"/>
+      <c r="D188" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A189" s="9"/>
+      <c r="C189" s="4"/>
+      <c r="D189" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A190" s="11"/>
+      <c r="B190" s="8"/>
+      <c r="C190" s="6"/>
+      <c r="D190" s="8"/>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A191" s="9"/>
+      <c r="C191" s="4"/>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A192" s="9">
         <v>4</v>
       </c>
-      <c r="C177" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D177" s="8" t="s">
+      <c r="C192" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D192" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A193" s="9"/>
+      <c r="C193" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D193" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A194" s="9"/>
+      <c r="C194" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D194" s="8"/>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A195" s="9"/>
+      <c r="C195" s="4"/>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A196" s="2">
+        <v>5</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D196" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C197" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D197" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C198" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D199" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D200" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A202" s="2">
+        <v>6</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C203" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D203" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C204" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A206" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B206" s="19"/>
+      <c r="C206" s="4"/>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A207" s="9">
+        <v>1</v>
+      </c>
+      <c r="C207" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D207" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A208" s="9"/>
+      <c r="C208" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D208" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A209" s="9"/>
+      <c r="C209" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D209" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A210" s="9"/>
+      <c r="C210" s="4"/>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A211" s="9">
+        <v>2</v>
+      </c>
+      <c r="C211" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D211" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A212" s="9"/>
+      <c r="C212" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D212" s="8" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C178" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="D178" s="8" t="s">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A213" s="9"/>
+      <c r="C213" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D213" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A215" s="2">
+        <v>3</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D215" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A216" s="8"/>
+      <c r="B216" s="8"/>
+      <c r="C216" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D216" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A217" s="8"/>
+      <c r="B217" s="8"/>
+      <c r="C217" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="D217" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A219" s="2">
+        <v>4</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D219" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C220" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D220" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C221" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D221" s="8"/>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A223" s="2">
+        <v>5</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C224" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="225" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C225" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D225" s="2" t="s">
         <v>185</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C179" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="D179" s="8"/>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A181" s="2">
-        <v>5</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D181" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C182" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D182" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C183" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D183" s="2" t="s">
-        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated user stories again
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A00329624\Documents\GitHub\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE47721-A6F1-4072-8EE8-FA3FC3676FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C72D2B-AFB7-4DEE-BBBE-BA432FC62095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
@@ -1238,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDD9AED8-E474-4BF9-9553-A6EDBA2E72AE}">
-  <dimension ref="A1:J225"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="2" customWidth="1"/>
@@ -3308,253 +3308,249 @@
       <c r="D190" s="8"/>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A191" s="9"/>
-      <c r="C191" s="4"/>
+      <c r="A191" s="9">
+        <v>3</v>
+      </c>
+      <c r="C191" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D191" s="8" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A192" s="9">
-        <v>4</v>
-      </c>
+      <c r="A192" s="9"/>
       <c r="C192" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D192" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="9"/>
       <c r="C193" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D193" s="8" t="s">
-        <v>124</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="D193" s="8"/>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="9"/>
-      <c r="C194" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D194" s="8"/>
+      <c r="C194" s="4"/>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A195" s="9"/>
-      <c r="C195" s="4"/>
+      <c r="A195" s="2">
+        <v>4</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A196" s="2">
-        <v>5</v>
-      </c>
       <c r="C196" s="2" t="s">
-        <v>125</v>
+        <v>186</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C197" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C198" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="D198" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D199" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D200" s="2" t="s">
         <v>192</v>
       </c>
     </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A201" s="2">
+        <v>5</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A202" s="2">
-        <v>6</v>
-      </c>
       <c r="C202" s="2" t="s">
-        <v>125</v>
+        <v>193</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C203" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C204" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D204" s="2" t="s">
         <v>197</v>
       </c>
     </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A205" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B205" s="19"/>
+      <c r="C205" s="4"/>
+    </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A206" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="B206" s="19"/>
-      <c r="C206" s="4"/>
-    </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A207" s="9">
+      <c r="A206" s="9">
         <v>1</v>
       </c>
+      <c r="C206" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D206" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A207" s="9"/>
       <c r="C207" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D207" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="208" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="9"/>
       <c r="C208" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D208" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="9"/>
-      <c r="C209" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="D209" s="8" t="s">
-        <v>144</v>
-      </c>
+      <c r="C209" s="4"/>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A210" s="9"/>
-      <c r="C210" s="4"/>
+      <c r="A210" s="9">
+        <v>2</v>
+      </c>
+      <c r="C210" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D210" s="8" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A211" s="9">
-        <v>2</v>
-      </c>
+      <c r="A211" s="9"/>
       <c r="C211" s="6" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D211" s="8" t="s">
-        <v>139</v>
+        <v>184</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="9"/>
       <c r="C212" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D212" s="8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A213" s="9"/>
-      <c r="C213" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D213" s="8" t="s">
         <v>145</v>
       </c>
     </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A214" s="2">
+        <v>3</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D214" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A215" s="2">
-        <v>3</v>
-      </c>
+      <c r="A215" s="8"/>
+      <c r="B215" s="8"/>
       <c r="C215" s="3" t="s">
-        <v>125</v>
+        <v>151</v>
       </c>
       <c r="D215" s="8" t="s">
-        <v>212</v>
+        <v>153</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="8"/>
       <c r="B216" s="8"/>
       <c r="C216" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D216" s="8" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A217" s="8"/>
-      <c r="B217" s="8"/>
-      <c r="C217" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="D217" s="8" t="s">
         <v>198</v>
       </c>
     </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A218" s="2">
+        <v>4</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D218" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A219" s="2">
-        <v>4</v>
-      </c>
       <c r="C219" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D219" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C220" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D220" s="8" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C221" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D221" s="8"/>
+      <c r="D220" s="8"/>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A222" s="2">
+        <v>5</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A223" s="2">
-        <v>5</v>
-      </c>
       <c r="C223" s="2" t="s">
-        <v>125</v>
+        <v>159</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C224" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="225" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C225" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="D225" s="2" t="s">
         <v>185</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Newsagent CREATE User Story
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a00327279\Downloads\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47381B0B-CD02-4F8C-AD48-CBA1F0D80CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEF4DF-0B92-45CD-9C5E-25AD1C5432A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="250">
   <si>
     <t>Number</t>
   </si>
@@ -766,6 +766,27 @@
   </si>
   <si>
     <t>I want to delete a newsagent</t>
+  </si>
+  <si>
+    <t>so that I have more managers</t>
+  </si>
+  <si>
+    <t>Verify that a valid(3 or more characters) Newsagent first name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(3 or more characters) Newsagent last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(10 numbers) Newsagent phone number can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if any Newsagent details entered are invalid, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the Newsagent is created</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the Newsagent is given a unique newsagent ID</t>
   </si>
 </sst>
 </file>
@@ -923,12 +944,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -950,6 +965,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1297,10 +1318,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
+      <c r="B1" s="30"/>
       <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
@@ -2033,7 +2054,7 @@
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="28" t="s">
+      <c r="A62" s="26" t="s">
         <v>3</v>
       </c>
       <c r="B62" s="17"/>
@@ -2422,7 +2443,7 @@
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="29" t="s">
+      <c r="A93" s="27" t="s">
         <v>61</v>
       </c>
       <c r="B93" s="18"/>
@@ -2826,7 +2847,7 @@
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="29" t="s">
+      <c r="A125" s="27" t="s">
         <v>90</v>
       </c>
       <c r="B125" s="18"/>
@@ -3044,7 +3065,7 @@
       <c r="C148" s="5"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="30" t="s">
+      <c r="A149" s="28" t="s">
         <v>108</v>
       </c>
       <c r="C149" s="5"/>
@@ -3266,7 +3287,7 @@
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" s="29" t="s">
+      <c r="A180" s="27" t="s">
         <v>134</v>
       </c>
       <c r="B180" s="18"/>
@@ -3450,7 +3471,7 @@
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A205" s="29" t="s">
+      <c r="A205" s="27" t="s">
         <v>89</v>
       </c>
       <c r="B205" s="18"/>
@@ -3615,31 +3636,31 @@
   <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="26" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="24" customWidth="1"/>
     <col min="2" max="2" width="1.7109375" customWidth="1"/>
     <col min="3" max="3" width="80.7109375" customWidth="1"/>
     <col min="4" max="4" width="185.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="21" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="25"/>
+      <c r="B2" s="23"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="26">
+      <c r="A3" s="24">
         <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -3696,7 +3717,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="26">
+      <c r="A12" s="24">
         <v>2</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -3735,7 +3756,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="26">
+      <c r="A18" s="24">
         <v>3</v>
       </c>
       <c r="C18" s="6" t="s">
@@ -3792,7 +3813,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="26">
+      <c r="A27" s="24">
         <v>4</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -3831,19 +3852,19 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="25" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="26">
+      <c r="A34" s="24">
         <v>1</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>221</v>
+        <v>244</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3851,41 +3872,40 @@
         <v>238</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>222</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C36" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D36" s="2"/>
+        <v>243</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>215</v>
+        <v>247</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C38" s="2"/>
       <c r="D38" s="2" t="s">
-        <v>223</v>
+        <v>248</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C39" s="5"/>
-      <c r="D39" s="2" t="s">
-        <v>21</v>
+      <c r="D39" s="8" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C40" s="5"/>
-      <c r="D40" s="2" t="s">
-        <v>178</v>
-      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="26">
+      <c r="A42" s="24">
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
@@ -3924,7 +3944,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="26">
+      <c r="A48" s="24">
         <v>3</v>
       </c>
       <c r="C48" s="1" t="s">
@@ -3981,7 +4001,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="26">
+      <c r="A57" s="24">
         <v>4</v>
       </c>
       <c r="C57" s="5" t="s">

</xml_diff>

<commit_message>
Update Project User Stories & Acceptance Criteria.xlsx
Updated all Newsagent User stories to match the project specifications, changed sheet one to list all entities, sheet 2 to completed entities that are currently being worked on.
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a00327279\Downloads\Software-Engineering-Project-G1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdthr\Downloads\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEF4DF-0B92-45CD-9C5E-25AD1C5432A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C8CD6F-8667-443E-A82D-5BD933BB4C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Entities" sheetId="1" r:id="rId1"/>
+    <sheet name="Completed User Stories" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="261">
   <si>
     <t>Number</t>
   </si>
@@ -759,9 +759,6 @@
     <t>I want to read a newsagent</t>
   </si>
   <si>
-    <t>so that I can view the information of a newsagent</t>
-  </si>
-  <si>
     <t>I want to update a newsagent</t>
   </si>
   <si>
@@ -771,22 +768,58 @@
     <t>so that I have more managers</t>
   </si>
   <si>
-    <t>Verify that a valid(3 or more characters) Newsagent first name can be entered</t>
-  </si>
-  <si>
-    <t>Verify that a valid(3 or more characters) Newsagent last name can be entered</t>
-  </si>
-  <si>
-    <t>Verify that a valid(10 numbers) Newsagent phone number can be entered</t>
-  </si>
-  <si>
-    <t>Verify that if any Newsagent details entered are invalid, an error message is returned</t>
-  </si>
-  <si>
-    <t>Verify that if all entered values are valid, the Newsagent is created</t>
-  </si>
-  <si>
-    <t>Verify that if all entered values are valid, the Newsagent is given a unique newsagent ID</t>
+    <t>so that I can view the information of another newsagent</t>
+  </si>
+  <si>
+    <t>Verify that a valid(10 numbers) newsagent phone number can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if any newsagent details entered are invalid, an error message is returned</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the newsagent is created</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the newsagent is given a unique newsagent ID</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) newsagent name can be entered to select the newsagent</t>
+  </si>
+  <si>
+    <t>Verify that the newsagent name is returned</t>
+  </si>
+  <si>
+    <t>Verify that the newsagent area code is returned</t>
+  </si>
+  <si>
+    <t>Verify that the newsagent phone number is returned</t>
+  </si>
+  <si>
+    <t>Verify that a customer can be selected by entering a valid customer ID, name, address, phone number or area code</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) newsagent ID, name, phone number can be entered to select the newsagent</t>
+  </si>
+  <si>
+    <t>Verify that a valid(1 or more characters) newsagent first name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(1 or more characters) newsagent last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that a valid(1 or more  characters) newsagent last name can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if all entered values are valid, the newsagent is updated</t>
+  </si>
+  <si>
+    <t>Verify that a valid(existing) newsagent ID, name, phone number can be entered</t>
+  </si>
+  <si>
+    <t>Verify that if the details entered is valid, the user is promted if they are sure they want to delete this newsagent from the database</t>
+  </si>
+  <si>
+    <t>Verify that if the user selects yes, the newsagent is removed</t>
   </si>
 </sst>
 </file>
@@ -882,7 +915,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -935,15 +968,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -970,6 +994,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1318,10 +1345,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
+      <c r="B1" s="27"/>
       <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
@@ -1330,10 +1357,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="16"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -2054,7 +2081,7 @@
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="26" t="s">
+      <c r="A62" s="23" t="s">
         <v>3</v>
       </c>
       <c r="B62" s="17"/>
@@ -2443,10 +2470,10 @@
       <c r="I92" s="1"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="27" t="s">
+      <c r="A93" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B93" s="18"/>
+      <c r="B93" s="16"/>
       <c r="C93" s="5"/>
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
@@ -2847,10 +2874,10 @@
       <c r="I124" s="1"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A125" s="27" t="s">
+      <c r="A125" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B125" s="18"/>
+      <c r="B125" s="16"/>
       <c r="C125" s="5"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
@@ -3065,7 +3092,7 @@
       <c r="C148" s="5"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="28" t="s">
+      <c r="A149" s="25" t="s">
         <v>108</v>
       </c>
       <c r="C149" s="5"/>
@@ -3287,10 +3314,10 @@
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" s="27" t="s">
+      <c r="A180" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="B180" s="18"/>
+      <c r="B180" s="16"/>
       <c r="C180" s="4"/>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
@@ -3471,10 +3498,10 @@
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A205" s="27" t="s">
+      <c r="A205" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="B205" s="18"/>
+      <c r="B205" s="16"/>
       <c r="C205" s="4"/>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
@@ -3633,34 +3660,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFD87129-AC48-47D3-BE6A-1FBC4D876D65}">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="24" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="21" customWidth="1"/>
     <col min="2" max="2" width="1.7109375" customWidth="1"/>
     <col min="3" max="3" width="80.7109375" customWidth="1"/>
     <col min="4" max="4" width="185.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="18" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="23"/>
+      <c r="B2" s="20"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="24">
+      <c r="A3" s="21">
         <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -3717,14 +3744,14 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="24">
+      <c r="A12" s="21">
         <v>2</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3756,7 +3783,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="24">
+      <c r="A18" s="21">
         <v>3</v>
       </c>
       <c r="C18" s="6" t="s">
@@ -3813,7 +3840,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="24">
+      <c r="A27" s="21">
         <v>4</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -3852,19 +3879,19 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="25" t="s">
+      <c r="A33" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="24">
+      <c r="A34" s="21">
         <v>1</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3872,47 +3899,47 @@
         <v>238</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C36" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C38" s="2"/>
       <c r="D38" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C39" s="5"/>
       <c r="D39" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C40" s="5"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="24">
+      <c r="A42" s="21">
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -3925,38 +3952,38 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C44" s="1" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>217</v>
+        <v>249</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C45" s="2"/>
       <c r="D45" s="2" t="s">
-        <v>216</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C46" s="2"/>
       <c r="D46" s="2" t="s">
-        <v>218</v>
+        <v>251</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="24">
+      <c r="A48" s="21">
         <v>3</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>220</v>
+        <v>253</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C49" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>72</v>
@@ -3967,76 +3994,344 @@
         <v>219</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>226</v>
+        <v>254</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C51" s="2"/>
       <c r="D51" s="2" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C52" s="2"/>
       <c r="D52" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C53" s="2"/>
       <c r="D53" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C54" s="2"/>
       <c r="D54" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C55" s="2"/>
-      <c r="D55" s="2" t="s">
-        <v>230</v>
+        <v>257</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="21">
+        <v>4</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="24">
-        <v>4</v>
-      </c>
       <c r="C57" s="5" t="s">
-        <v>4</v>
+        <v>241</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C58" s="5" t="s">
-        <v>242</v>
+        <v>23</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>225</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C59" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="C59" s="5"/>
       <c r="D59" s="2" t="s">
-        <v>24</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C60" s="5"/>
       <c r="D60" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C61" s="5"/>
-      <c r="D61" s="2" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" s="16"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="2"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="9">
+        <v>1</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="9"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="9"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="9"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="9"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="9"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="9"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="2"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="9">
+        <v>2</v>
+      </c>
+      <c r="B70" s="2"/>
+      <c r="C70" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="9"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="9"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="9"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="9"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="9"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="5"/>
+      <c r="D75" s="2"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="9">
+        <v>3</v>
+      </c>
+      <c r="B76" s="2"/>
+      <c r="C76" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="9"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="9"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="9"/>
+      <c r="B79" s="2"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="9"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="9"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" s="9"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="5"/>
+      <c r="D82" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="9"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="9"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="5"/>
+      <c r="D84" s="2"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="9">
+        <v>4</v>
+      </c>
+      <c r="B85" s="2"/>
+      <c r="C85" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D85" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="9"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="9"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="9"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="5"/>
+      <c r="D88" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="9"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="9"/>
+      <c r="B90" s="2"/>
+      <c r="C90" s="5"/>
+      <c r="D90" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="9"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="5"/>
+      <c r="D91" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92" s="9"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="5"/>
+      <c r="D92" s="8" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed outdated files & Changed Plan Increments
</commit_message>
<xml_diff>
--- a/Project User Stories & Acceptance Criteria.xlsx
+++ b/Project User Stories & Acceptance Criteria.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdthr\Downloads\Software-Engineering-Project-G1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TEMP.TUSSTUDENT.023\Downloads\Software-Engineering-Project-G1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F7378F-33A2-428C-8833-553E61A9822A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D8C0F2E-504E-4D73-8FB9-107926871AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5F9D763-E16F-42A4-9C71-431260985051}"/>
   </bookViews>
@@ -32,12 +32,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="245">
   <si>
     <t>Number</t>
   </si>
@@ -754,6 +757,24 @@
   </si>
   <si>
     <t>Verify that if the user selects yes, the newsagent is removed</t>
+  </si>
+  <si>
+    <t>I want to create a delivery person</t>
+  </si>
+  <si>
+    <t>so that I have more deliveries to customers</t>
+  </si>
+  <si>
+    <t>I want to read a delivery person</t>
+  </si>
+  <si>
+    <t>so that I can view the information of the delivery person</t>
+  </si>
+  <si>
+    <t>I want to update a delivery person</t>
+  </si>
+  <si>
+    <t>I want to delete a delivery person</t>
   </si>
 </sst>
 </file>
@@ -808,7 +829,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -824,6 +845,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -849,7 +876,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -930,6 +957,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1774,7 +1808,7 @@
       <c r="I38" s="1"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="28" t="s">
         <v>31</v>
       </c>
       <c r="B39" s="16"/>
@@ -3622,7 +3656,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFD87129-AC48-47D3-BE6A-1FBC4D876D65}">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" style="21" customWidth="1"/>
@@ -4173,27 +4207,27 @@
         <v>4</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="9"/>
       <c r="B79" s="2"/>
       <c r="C79" s="5" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="9"/>
       <c r="B80" s="2"/>
       <c r="C80" s="5" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -4201,77 +4235,75 @@
       <c r="B81" s="2"/>
       <c r="C81" s="5"/>
       <c r="D81" s="8" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="9"/>
       <c r="B82" s="2"/>
       <c r="C82" s="5"/>
-      <c r="D82" s="8" t="s">
-        <v>23</v>
+      <c r="D82" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="9"/>
       <c r="B83" s="2"/>
       <c r="C83" s="5"/>
-      <c r="D83" s="2"/>
+      <c r="D83" s="2" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="9">
-        <v>3</v>
-      </c>
+      <c r="A84" s="9"/>
       <c r="B84" s="2"/>
-      <c r="C84" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="C84" s="5"/>
       <c r="D84" s="8" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
       <c r="B85" s="2"/>
-      <c r="C85" s="5" t="s">
-        <v>70</v>
-      </c>
+      <c r="C85" s="5"/>
       <c r="D85" s="8" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
       <c r="B86" s="2"/>
-      <c r="C86" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="9"/>
+      <c r="A87" s="9">
+        <v>3</v>
+      </c>
       <c r="B87" s="2"/>
-      <c r="C87" s="5"/>
+      <c r="C87" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D87" s="8" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
       <c r="B88" s="2"/>
-      <c r="C88" s="5"/>
+      <c r="C88" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="D88" s="8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
       <c r="B89" s="2"/>
-      <c r="C89" s="5"/>
+      <c r="C89" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="D89" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -4279,7 +4311,7 @@
       <c r="B90" s="2"/>
       <c r="C90" s="5"/>
       <c r="D90" s="8" t="s">
-        <v>74</v>
+        <v>23</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -4287,69 +4319,67 @@
       <c r="B91" s="2"/>
       <c r="C91" s="5"/>
       <c r="D91" s="8" t="s">
-        <v>175</v>
+        <v>73</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
       <c r="B92" s="2"/>
       <c r="C92" s="5"/>
-      <c r="D92" s="2"/>
+      <c r="D92" s="8" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="9">
-        <v>4</v>
-      </c>
+      <c r="A93" s="9"/>
       <c r="B93" s="2"/>
-      <c r="C93" s="5" t="s">
-        <v>4</v>
-      </c>
+      <c r="C93" s="5"/>
       <c r="D93" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="9"/>
       <c r="B94" s="2"/>
-      <c r="C94" s="5" t="s">
-        <v>75</v>
-      </c>
+      <c r="C94" s="5"/>
       <c r="D94" s="8" t="s">
-        <v>78</v>
+        <v>175</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
       <c r="B95" s="2"/>
-      <c r="C95" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D95" s="8" t="s">
-        <v>79</v>
-      </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="9"/>
+      <c r="A96" s="9">
+        <v>4</v>
+      </c>
       <c r="B96" s="2"/>
-      <c r="C96" s="5"/>
+      <c r="C96" s="5" t="s">
+        <v>4</v>
+      </c>
       <c r="D96" s="8" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="9"/>
       <c r="B97" s="2"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="2" t="s">
-        <v>81</v>
+      <c r="C97" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D97" s="8" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="9"/>
       <c r="B98" s="2"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="2" t="s">
-        <v>82</v>
+      <c r="C98" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D98" s="8" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4357,7 +4387,7 @@
       <c r="B99" s="2"/>
       <c r="C99" s="5"/>
       <c r="D99" s="8" t="s">
-        <v>83</v>
+        <v>174</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4365,7 +4395,190 @@
       <c r="B100" s="2"/>
       <c r="C100" s="5"/>
       <c r="D100" s="8" t="s">
-        <v>84</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D102" s="30"/>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" s="21">
+        <v>1</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="2"/>
+      <c r="D106" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="2"/>
+      <c r="D107" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="5"/>
+      <c r="D108" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C109" s="5"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" s="21">
+        <v>2</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C111" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C112" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C113" s="2"/>
+      <c r="D113" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C114" s="2"/>
+      <c r="D114" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="21">
+        <v>3</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C117" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C118" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C119" s="2"/>
+      <c r="D119" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C120" s="2"/>
+      <c r="D120" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C121" s="2"/>
+      <c r="D121" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C122" s="2"/>
+      <c r="D122" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="21">
+        <v>4</v>
+      </c>
+      <c r="C124" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C125" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C126" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C127" s="5"/>
+      <c r="D127" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C128" s="5"/>
+      <c r="D128" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>